<commit_message>
Corrigido filtro estrito de meses: nenhuma despesa passada vaza para outros meses
</commit_message>
<xml_diff>
--- a/Controle_Financeiro_2026.xlsx
+++ b/Controle_Financeiro_2026.xlsx
@@ -1593,7 +1593,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:H76"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2140,6 +2140,9 @@
       </c>
     </row>
     <row r="28">
+      <c r="A28" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="B28">
         <v>46265</v>
       </c>
@@ -2151,13 +2154,16 @@
       </c>
     </row>
     <row r="29">
-      <c r="J29" t="str">
-        <v>🛑Atrasado</v>
+      <c r="A29" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -2165,7 +2171,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Custos Variáveis</v>
+        <v>Impostos e Taxas</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -2173,7 +2179,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Impostos e Taxas</v>
+        <v>Pró-labore / Retirada</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -2181,10 +2187,28 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Pró-labore / Retirada</v>
+        <v>Agosto</v>
+      </c>
+      <c r="B33">
+        <v>46239</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Deal Suporte e Tecnologia</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>300</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Filmagem</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Entregue</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Não emitida</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Parcela 1/2</v>
       </c>
     </row>
     <row r="34">
@@ -2192,13 +2216,13 @@
         <v>Agosto</v>
       </c>
       <c r="B34">
-        <v>46239</v>
+        <v>46244</v>
       </c>
       <c r="C34" t="str">
         <v>Deal Suporte e Tecnologia</v>
       </c>
       <c r="D34">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="E34" t="str">
         <v>Filmagem</v>
@@ -2210,7 +2234,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H34" t="str">
-        <v>Parcela 1/2</v>
+        <v>Parcela 2/2</v>
       </c>
     </row>
     <row r="35">
@@ -2221,22 +2245,22 @@
         <v>46244</v>
       </c>
       <c r="C35" t="str">
-        <v>Deal Suporte e Tecnologia</v>
+        <v>Quinto Andar (GRPQA LTDA)</v>
       </c>
       <c r="D35">
-        <v>200</v>
+        <v>1472.09</v>
       </c>
       <c r="E35" t="str">
-        <v>Filmagem</v>
+        <v>Quinto Andar</v>
       </c>
       <c r="F35" t="str">
         <v>Entregue</v>
       </c>
       <c r="G35" t="str">
-        <v>Não emitida</v>
+        <v>Não se aplica</v>
       </c>
       <c r="H35" t="str">
-        <v>Parcela 2/2</v>
+        <v>Renda de aluguel recebida na PF</v>
       </c>
     </row>
     <row r="36">
@@ -2244,25 +2268,25 @@
         <v>Agosto</v>
       </c>
       <c r="B36">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="C36" t="str">
-        <v>Quinto Andar (GRPQA LTDA)</v>
+        <v>GBF Nutri LTDA-ME</v>
       </c>
       <c r="D36">
-        <v>1472.09</v>
+        <v>1400</v>
       </c>
       <c r="E36" t="str">
-        <v>Quinto Andar</v>
+        <v>Filmagem</v>
       </c>
       <c r="F36" t="str">
-        <v>Entregue</v>
+        <v>Não Entregue</v>
       </c>
       <c r="G36" t="str">
-        <v>Não se aplica</v>
+        <v>Não emitida</v>
       </c>
       <c r="H36" t="str">
-        <v>Renda de aluguel recebida na PF</v>
+        <v>Evento Gabriela Nutri - Cobertura Vídeo e Foto</v>
       </c>
     </row>
     <row r="37">
@@ -2270,13 +2294,13 @@
         <v>Agosto</v>
       </c>
       <c r="B37">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C37" t="str">
-        <v>GBF Nutri LTDA-ME</v>
+        <v>Elisa Jardim (Velocity)</v>
       </c>
       <c r="D37">
-        <v>1400</v>
+        <v>225</v>
       </c>
       <c r="E37" t="str">
         <v>Filmagem</v>
@@ -2288,7 +2312,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H37" t="str">
-        <v>Evento Gabriela Nutri - Cobertura Vídeo e Foto</v>
+        <v>Cobertura Aniversário Velocity - Parcela 1/2</v>
       </c>
     </row>
     <row r="38">
@@ -2296,25 +2320,25 @@
         <v>Agosto</v>
       </c>
       <c r="B38">
-        <v>46248</v>
+        <v>46250</v>
       </c>
       <c r="C38" t="str">
-        <v>Elisa Jardim (Velocity)</v>
+        <v>Letras e Cia Assessoria (Amigo)</v>
       </c>
       <c r="D38">
-        <v>225</v>
+        <v>200</v>
       </c>
       <c r="E38" t="str">
-        <v>Filmagem</v>
+        <v>Outros</v>
       </c>
       <c r="F38" t="str">
-        <v>Não Entregue</v>
+        <v>Entregue</v>
       </c>
       <c r="G38" t="str">
-        <v>Não emitida</v>
+        <v>Não se aplica</v>
       </c>
       <c r="H38" t="str">
-        <v>Cobertura Aniversário Velocity - Parcela 1/2</v>
+        <v>Entrada Pessoal (transferência de amigo via PF)</v>
       </c>
     </row>
     <row r="39">
@@ -2322,25 +2346,25 @@
         <v>Agosto</v>
       </c>
       <c r="B39">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C39" t="str">
-        <v>Letras e Cia Assessoria (Amigo)</v>
+        <v>Mariana Borges Retamoso</v>
       </c>
       <c r="D39">
-        <v>200</v>
+        <v>550</v>
       </c>
       <c r="E39" t="str">
-        <v>Outros</v>
+        <v>Fotografia</v>
       </c>
       <c r="F39" t="str">
-        <v>Entregue</v>
+        <v>Não Entregue</v>
       </c>
       <c r="G39" t="str">
-        <v>Não se aplica</v>
+        <v>Não emitida</v>
       </c>
       <c r="H39" t="str">
-        <v>Entrada Pessoal (transferência de amigo via PF)</v>
+        <v>Pacote 20 Fotos Grumari - Parcela 1/2</v>
       </c>
     </row>
     <row r="40">
@@ -2351,13 +2375,13 @@
         <v>46251</v>
       </c>
       <c r="C40" t="str">
-        <v>Mariana Borges Retamoso</v>
+        <v>Paula Cristina (Projeto Maris)</v>
       </c>
       <c r="D40">
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="E40" t="str">
-        <v>Fotografia</v>
+        <v>Filmagem</v>
       </c>
       <c r="F40" t="str">
         <v>Não Entregue</v>
@@ -2366,7 +2390,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H40" t="str">
-        <v>Pacote 20 Fotos Grumari - Parcela 1/2</v>
+        <v>Cobertura Vídeo Fórum ANB</v>
       </c>
     </row>
     <row r="41">
@@ -2374,13 +2398,13 @@
         <v>Agosto</v>
       </c>
       <c r="B41">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C41" t="str">
-        <v>Paula Cristina (Projeto Maris)</v>
+        <v>Tatiana Sampaio</v>
       </c>
       <c r="D41">
-        <v>500</v>
+        <v>2200</v>
       </c>
       <c r="E41" t="str">
         <v>Filmagem</v>
@@ -2392,7 +2416,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H41" t="str">
-        <v>Cobertura Vídeo Fórum ANB</v>
+        <v>Pacote Vertical 10 / Vídeos</v>
       </c>
     </row>
     <row r="42">
@@ -2400,13 +2424,13 @@
         <v>Agosto</v>
       </c>
       <c r="B42">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C42" t="str">
-        <v>Tatiana Sampaio</v>
+        <v>Irmãos Caxeiros Lanchonete</v>
       </c>
       <c r="D42">
-        <v>2200</v>
+        <v>625</v>
       </c>
       <c r="E42" t="str">
         <v>Filmagem</v>
@@ -2418,7 +2442,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H42" t="str">
-        <v>Pacote Vertical 10 / Vídeos</v>
+        <v>Filmagem / Social Media</v>
       </c>
     </row>
     <row r="43">
@@ -2426,25 +2450,25 @@
         <v>Agosto</v>
       </c>
       <c r="B43">
-        <v>46253</v>
+        <v>46258</v>
       </c>
       <c r="C43" t="str">
-        <v>Irmãos Caxeiros Lanchonete</v>
+        <v>Giovanni Santos de Souza</v>
       </c>
       <c r="D43">
-        <v>625</v>
+        <v>312</v>
       </c>
       <c r="E43" t="str">
-        <v>Filmagem</v>
+        <v>Fotografia</v>
       </c>
       <c r="F43" t="str">
-        <v>Não Entregue</v>
+        <v>Entregue</v>
       </c>
       <c r="G43" t="str">
         <v>Não emitida</v>
       </c>
       <c r="H43" t="str">
-        <v>Filmagem / Social Media</v>
+        <v>Pix recebido via PF - Parcela 1/2</v>
       </c>
     </row>
     <row r="44">
@@ -2452,25 +2476,25 @@
         <v>Agosto</v>
       </c>
       <c r="B44">
-        <v>46258</v>
+        <v>46261</v>
       </c>
       <c r="C44" t="str">
-        <v>Giovanni Santos de Souza</v>
+        <v>Espaço VIP / Edson Açai Gourmet</v>
       </c>
       <c r="D44">
-        <v>312</v>
+        <v>1250</v>
       </c>
       <c r="E44" t="str">
-        <v>Fotografia</v>
+        <v>Filmagem</v>
       </c>
       <c r="F44" t="str">
-        <v>Entregue</v>
+        <v>Não Entregue</v>
       </c>
       <c r="G44" t="str">
         <v>Não emitida</v>
       </c>
       <c r="H44" t="str">
-        <v>Pix recebido via PF - Parcela 1/2</v>
+        <v>Meta Ads e Vídeos para loja</v>
       </c>
     </row>
     <row r="45">
@@ -2478,25 +2502,25 @@
         <v>Agosto</v>
       </c>
       <c r="B45">
-        <v>46261</v>
+        <v>46264</v>
       </c>
       <c r="C45" t="str">
-        <v>Espaço VIP / Edson Açai Gourmet</v>
+        <v>Giovanni Santos de Souza</v>
       </c>
       <c r="D45">
-        <v>1250</v>
+        <v>100</v>
       </c>
       <c r="E45" t="str">
-        <v>Filmagem</v>
+        <v>Fotografia</v>
       </c>
       <c r="F45" t="str">
-        <v>Não Entregue</v>
+        <v>Entregue</v>
       </c>
       <c r="G45" t="str">
         <v>Não emitida</v>
       </c>
       <c r="H45" t="str">
-        <v>Meta Ads e Vídeos para loja</v>
+        <v>Pix recebido via PF - Parcela 2/2</v>
       </c>
     </row>
     <row r="46">
@@ -2504,16 +2528,16 @@
         <v>Agosto</v>
       </c>
       <c r="B46">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="C46" t="str">
-        <v>Giovanni Santos de Souza</v>
+        <v>Roberta Simões de Oliveira</v>
       </c>
       <c r="D46">
-        <v>100</v>
+        <v>700</v>
       </c>
       <c r="E46" t="str">
-        <v>Fotografia</v>
+        <v>Filmagem</v>
       </c>
       <c r="F46" t="str">
         <v>Entregue</v>
@@ -2522,7 +2546,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H46" t="str">
-        <v>Pix recebido via PF - Parcela 2/2</v>
+        <v>Pix recebido via PF</v>
       </c>
     </row>
     <row r="47">
@@ -2533,48 +2557,48 @@
         <v>46265</v>
       </c>
       <c r="C47" t="str">
-        <v>Roberta Simões de Oliveira</v>
+        <v>Davi Araújo da Silva</v>
       </c>
       <c r="D47">
-        <v>700</v>
+        <v>850</v>
       </c>
       <c r="E47" t="str">
         <v>Filmagem</v>
       </c>
       <c r="F47" t="str">
-        <v>Entregue</v>
+        <v>Não Entregue</v>
       </c>
       <c r="G47" t="str">
         <v>Não emitida</v>
       </c>
       <c r="H47" t="str">
-        <v>Pix recebido via PF</v>
+        <v>Serviços Audiovisuais</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Agosto</v>
+        <v>Junho</v>
       </c>
       <c r="B48">
-        <v>46265</v>
+        <v>46174</v>
       </c>
       <c r="C48" t="str">
-        <v>Davi Araújo da Silva</v>
+        <v>Débora Renata Olibano Ribeiro</v>
       </c>
       <c r="D48">
-        <v>850</v>
+        <v>1500</v>
       </c>
       <c r="E48" t="str">
         <v>Filmagem</v>
       </c>
       <c r="F48" t="str">
-        <v>Não Entregue</v>
+        <v>Entregue</v>
       </c>
       <c r="G48" t="str">
         <v>Não emitida</v>
       </c>
       <c r="H48" t="str">
-        <v>Serviços Audiovisuais</v>
+        <v>Pix recebido via PJ</v>
       </c>
     </row>
     <row r="49">
@@ -2582,13 +2606,13 @@
         <v>Junho</v>
       </c>
       <c r="B49">
-        <v>46174</v>
+        <v>46177</v>
       </c>
       <c r="C49" t="str">
-        <v>Débora Renata Olibano Ribeiro</v>
+        <v>Antonio Carlos Barbeito Mendes</v>
       </c>
       <c r="D49">
-        <v>1500</v>
+        <v>1300</v>
       </c>
       <c r="E49" t="str">
         <v>Filmagem</v>
@@ -2608,13 +2632,13 @@
         <v>Junho</v>
       </c>
       <c r="B50">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="C50" t="str">
-        <v>Antonio Carlos Barbeito Mendes</v>
+        <v>Anderson Coutinho Paleologo</v>
       </c>
       <c r="D50">
-        <v>1300</v>
+        <v>486.8</v>
       </c>
       <c r="E50" t="str">
         <v>Filmagem</v>
@@ -2634,25 +2658,25 @@
         <v>Junho</v>
       </c>
       <c r="B51">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="C51" t="str">
-        <v>Anderson Coutinho Paleologo</v>
+        <v>GRPQA LTDA (Quinto Andar)</v>
       </c>
       <c r="D51">
-        <v>486.8</v>
+        <v>1472.09</v>
       </c>
       <c r="E51" t="str">
-        <v>Filmagem</v>
+        <v>Quinto Andar</v>
       </c>
       <c r="F51" t="str">
         <v>Entregue</v>
       </c>
       <c r="G51" t="str">
-        <v>Não emitida</v>
+        <v>Não se aplica</v>
       </c>
       <c r="H51" t="str">
-        <v>Pix recebido via PJ</v>
+        <v>Renda de aluguel recebida na PF</v>
       </c>
     </row>
     <row r="52">
@@ -2660,25 +2684,25 @@
         <v>Junho</v>
       </c>
       <c r="B52">
-        <v>46182</v>
+        <v>46187</v>
       </c>
       <c r="C52" t="str">
-        <v>GRPQA LTDA (Quinto Andar)</v>
+        <v>Silvia Bretz (via iFood Pago)</v>
       </c>
       <c r="D52">
-        <v>1472.09</v>
+        <v>5250</v>
       </c>
       <c r="E52" t="str">
-        <v>Quinto Andar</v>
+        <v>Filmagem</v>
       </c>
       <c r="F52" t="str">
         <v>Entregue</v>
       </c>
       <c r="G52" t="str">
-        <v>Não se aplica</v>
+        <v>Não emitida</v>
       </c>
       <c r="H52" t="str">
-        <v>Renda de aluguel recebida na PF</v>
+        <v>Filmagem Silvia Bretz - Contrato Audiovisual</v>
       </c>
     </row>
     <row r="53">
@@ -2686,25 +2710,25 @@
         <v>Junho</v>
       </c>
       <c r="B53">
-        <v>46187</v>
+        <v>46192</v>
       </c>
       <c r="C53" t="str">
-        <v>Silvia Bretz (via iFood Pago)</v>
+        <v>Andrea Fernandes Guimarães</v>
       </c>
       <c r="D53">
-        <v>5250</v>
+        <v>500</v>
       </c>
       <c r="E53" t="str">
-        <v>Filmagem</v>
+        <v>Apoio / Outros</v>
       </c>
       <c r="F53" t="str">
         <v>Entregue</v>
       </c>
       <c r="G53" t="str">
-        <v>Não emitida</v>
+        <v>Não se aplica</v>
       </c>
       <c r="H53" t="str">
-        <v>Filmagem Silvia Bretz - Contrato Audiovisual</v>
+        <v>Repasse / Devolução</v>
       </c>
     </row>
     <row r="54">
@@ -2712,7 +2736,7 @@
         <v>Junho</v>
       </c>
       <c r="B54">
-        <v>46192</v>
+        <v>46196</v>
       </c>
       <c r="C54" t="str">
         <v>Andrea Fernandes Guimarães</v>
@@ -2738,25 +2762,25 @@
         <v>Junho</v>
       </c>
       <c r="B55">
-        <v>46196</v>
+        <v>46199</v>
       </c>
       <c r="C55" t="str">
-        <v>Andrea Fernandes Guimarães</v>
+        <v>Edinaldo Dalcin de Souza</v>
       </c>
       <c r="D55">
         <v>500</v>
       </c>
       <c r="E55" t="str">
-        <v>Apoio / Outros</v>
+        <v>Filmagem</v>
       </c>
       <c r="F55" t="str">
         <v>Entregue</v>
       </c>
       <c r="G55" t="str">
-        <v>Não se aplica</v>
+        <v>Não emitida</v>
       </c>
       <c r="H55" t="str">
-        <v>Repasse / Devolução</v>
+        <v>Pix recebido via PJ</v>
       </c>
     </row>
     <row r="56">
@@ -2764,25 +2788,25 @@
         <v>Junho</v>
       </c>
       <c r="B56">
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="C56" t="str">
-        <v>Edinaldo Dalcin de Souza</v>
+        <v>Andrea Fernandes Guimarães</v>
       </c>
       <c r="D56">
         <v>500</v>
       </c>
       <c r="E56" t="str">
-        <v>Filmagem</v>
+        <v>Apoio / Outros</v>
       </c>
       <c r="F56" t="str">
         <v>Entregue</v>
       </c>
       <c r="G56" t="str">
-        <v>Não emitida</v>
+        <v>Não se aplica</v>
       </c>
       <c r="H56" t="str">
-        <v>Pix recebido via PJ</v>
+        <v>Repasse / Devolução</v>
       </c>
     </row>
     <row r="57">
@@ -2790,39 +2814,39 @@
         <v>Junho</v>
       </c>
       <c r="B57">
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="C57" t="str">
-        <v>Andrea Fernandes Guimarães</v>
+        <v>Fernanda Palmeira L Moreira</v>
       </c>
       <c r="D57">
-        <v>500</v>
+        <v>825</v>
       </c>
       <c r="E57" t="str">
-        <v>Apoio / Outros</v>
+        <v>Filmagem</v>
       </c>
       <c r="F57" t="str">
         <v>Entregue</v>
       </c>
       <c r="G57" t="str">
-        <v>Não se aplica</v>
+        <v>Não emitida</v>
       </c>
       <c r="H57" t="str">
-        <v>Repasse / Devolução</v>
+        <v>Parcela 1/2</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Junho</v>
+        <v>Julho</v>
       </c>
       <c r="B58">
-        <v>46203</v>
+        <v>46206</v>
       </c>
       <c r="C58" t="str">
-        <v>Fernanda Palmeira L Moreira</v>
+        <v>Thiago de Santa Martha dos Santos</v>
       </c>
       <c r="D58">
-        <v>825</v>
+        <v>700</v>
       </c>
       <c r="E58" t="str">
         <v>Filmagem</v>
@@ -2834,7 +2858,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H58" t="str">
-        <v>Parcela 1/2</v>
+        <v>Pix recebido via PJ</v>
       </c>
     </row>
     <row r="59">
@@ -2842,13 +2866,13 @@
         <v>Julho</v>
       </c>
       <c r="B59">
-        <v>46206</v>
+        <v>46212</v>
       </c>
       <c r="C59" t="str">
-        <v>Thiago de Santa Martha dos Santos</v>
+        <v>Fernanda Palmeira L Moreira</v>
       </c>
       <c r="D59">
-        <v>700</v>
+        <v>825</v>
       </c>
       <c r="E59" t="str">
         <v>Filmagem</v>
@@ -2860,7 +2884,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H59" t="str">
-        <v>Pix recebido via PJ</v>
+        <v>Parcela 2/2</v>
       </c>
     </row>
     <row r="60">
@@ -2874,7 +2898,7 @@
         <v>Fernanda Palmeira L Moreira</v>
       </c>
       <c r="D60">
-        <v>825</v>
+        <v>100</v>
       </c>
       <c r="E60" t="str">
         <v>Filmagem</v>
@@ -2886,7 +2910,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H60" t="str">
-        <v>Parcela 2/2</v>
+        <v>Adicional / Taxa</v>
       </c>
     </row>
     <row r="61">
@@ -2894,25 +2918,25 @@
         <v>Julho</v>
       </c>
       <c r="B61">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="C61" t="str">
-        <v>Fernanda Palmeira L Moreira</v>
+        <v>GRPQA LTDA (Quinto Andar)</v>
       </c>
       <c r="D61">
-        <v>100</v>
+        <v>1472.09</v>
       </c>
       <c r="E61" t="str">
-        <v>Filmagem</v>
+        <v>Quinto Andar</v>
       </c>
       <c r="F61" t="str">
         <v>Entregue</v>
       </c>
       <c r="G61" t="str">
-        <v>Não emitida</v>
+        <v>Não se aplica</v>
       </c>
       <c r="H61" t="str">
-        <v>Adicional / Taxa</v>
+        <v>Renda de aluguel recebida na PF</v>
       </c>
     </row>
     <row r="62">
@@ -2920,25 +2944,25 @@
         <v>Julho</v>
       </c>
       <c r="B62">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="C62" t="str">
-        <v>GRPQA LTDA (Quinto Andar)</v>
+        <v>Tree Intelligence Soluções Tecnológicas</v>
       </c>
       <c r="D62">
-        <v>1472.09</v>
+        <v>450</v>
       </c>
       <c r="E62" t="str">
-        <v>Quinto Andar</v>
+        <v>Filmagem</v>
       </c>
       <c r="F62" t="str">
         <v>Entregue</v>
       </c>
       <c r="G62" t="str">
-        <v>Não se aplica</v>
+        <v>Não emitida</v>
       </c>
       <c r="H62" t="str">
-        <v>Renda de aluguel recebida na PF</v>
+        <v>Pix recebido via PJ</v>
       </c>
     </row>
     <row r="63">
@@ -2946,16 +2970,16 @@
         <v>Julho</v>
       </c>
       <c r="B63">
-        <v>46217</v>
+        <v>46224</v>
       </c>
       <c r="C63" t="str">
-        <v>Tree Intelligence Soluções Tecnológicas</v>
+        <v>Alexandre Juncken Antiguidades</v>
       </c>
       <c r="D63">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="E63" t="str">
-        <v>Filmagem</v>
+        <v>Fotografia</v>
       </c>
       <c r="F63" t="str">
         <v>Entregue</v>
@@ -2972,16 +2996,16 @@
         <v>Julho</v>
       </c>
       <c r="B64">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="C64" t="str">
-        <v>Alexandre Juncken Antiguidades</v>
+        <v>Cintia de Brito Barreto Saldanha</v>
       </c>
       <c r="D64">
-        <v>100</v>
+        <v>800</v>
       </c>
       <c r="E64" t="str">
-        <v>Fotografia</v>
+        <v>Filmagem</v>
       </c>
       <c r="F64" t="str">
         <v>Entregue</v>
@@ -2990,7 +3014,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H64" t="str">
-        <v>Pix recebido via PJ</v>
+        <v>Cobertura Vídeo</v>
       </c>
     </row>
     <row r="65">
@@ -3001,22 +3025,22 @@
         <v>46227</v>
       </c>
       <c r="C65" t="str">
-        <v>Cintia de Brito Barreto Saldanha</v>
+        <v>Letras e Cia Assessoria (Amigo)</v>
       </c>
       <c r="D65">
-        <v>800</v>
+        <v>150</v>
       </c>
       <c r="E65" t="str">
-        <v>Filmagem</v>
+        <v>Outros</v>
       </c>
       <c r="F65" t="str">
         <v>Entregue</v>
       </c>
       <c r="G65" t="str">
-        <v>Não emitida</v>
+        <v>Não se aplica</v>
       </c>
       <c r="H65" t="str">
-        <v>Cobertura Vídeo</v>
+        <v>Entrada Pessoal (transferência de amigo via PF)</v>
       </c>
     </row>
     <row r="66">
@@ -3027,22 +3051,22 @@
         <v>46227</v>
       </c>
       <c r="C66" t="str">
-        <v>Letras e Cia Assessoria (Amigo)</v>
+        <v>Vendas Cartão (InfinitePay / CloudWalk)</v>
       </c>
       <c r="D66">
-        <v>150</v>
+        <v>756</v>
       </c>
       <c r="E66" t="str">
-        <v>Outros</v>
+        <v>Filmagem</v>
       </c>
       <c r="F66" t="str">
         <v>Entregue</v>
       </c>
       <c r="G66" t="str">
-        <v>Não se aplica</v>
+        <v>Não emitida</v>
       </c>
       <c r="H66" t="str">
-        <v>Entrada Pessoal (transferência de amigo via PF)</v>
+        <v>Recebimento maquininha</v>
       </c>
     </row>
     <row r="67">
@@ -3050,13 +3074,13 @@
         <v>Julho</v>
       </c>
       <c r="B67">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C67" t="str">
-        <v>Vendas Cartão (InfinitePay / CloudWalk)</v>
+        <v>GBF Nutri LTDA-ME</v>
       </c>
       <c r="D67">
-        <v>756</v>
+        <v>1400</v>
       </c>
       <c r="E67" t="str">
         <v>Filmagem</v>
@@ -3068,7 +3092,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H67" t="str">
-        <v>Recebimento maquininha</v>
+        <v>Evento Gabi Nutri - Cobertura 1/2</v>
       </c>
     </row>
     <row r="68">
@@ -3076,13 +3100,13 @@
         <v>Julho</v>
       </c>
       <c r="B68">
-        <v>46228</v>
+        <v>46231</v>
       </c>
       <c r="C68" t="str">
-        <v>GBF Nutri LTDA-ME</v>
+        <v>Julio Cesar de Araujo</v>
       </c>
       <c r="D68">
-        <v>1400</v>
+        <v>2000</v>
       </c>
       <c r="E68" t="str">
         <v>Filmagem</v>
@@ -3094,7 +3118,7 @@
         <v>Não emitida</v>
       </c>
       <c r="H68" t="str">
-        <v>Evento Gabi Nutri - Cobertura 1/2</v>
+        <v>Produção Audiovisual</v>
       </c>
     </row>
     <row r="69">
@@ -3105,10 +3129,10 @@
         <v>46231</v>
       </c>
       <c r="C69" t="str">
-        <v>Julio Cesar de Araujo</v>
+        <v>Forja Segurança Eletrônica</v>
       </c>
       <c r="D69">
-        <v>2000</v>
+        <v>50</v>
       </c>
       <c r="E69" t="str">
         <v>Filmagem</v>
@@ -3120,33 +3144,15 @@
         <v>Não emitida</v>
       </c>
       <c r="H69" t="str">
-        <v>Produção Audiovisual</v>
+        <v>Serviço Audiovisual</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Julho</v>
-      </c>
-      <c r="B70">
-        <v>46231</v>
-      </c>
-      <c r="C70" t="str">
-        <v>Forja Segurança Eletrônica</v>
+        <v>Total</v>
       </c>
       <c r="D70">
-        <v>50</v>
-      </c>
-      <c r="E70" t="str">
-        <v>Filmagem</v>
-      </c>
-      <c r="F70" t="str">
-        <v>Entregue</v>
-      </c>
-      <c r="G70" t="str">
-        <v>Não emitida</v>
-      </c>
-      <c r="H70" t="str">
-        <v>Serviço Audiovisual</v>
+        <v>5740.59</v>
       </c>
     </row>
     <row r="71">
@@ -3154,7 +3160,7 @@
         <v>Total</v>
       </c>
       <c r="D71">
-        <v>5740.59</v>
+        <v>4100</v>
       </c>
     </row>
     <row r="72">
@@ -3162,7 +3168,7 @@
         <v>Total</v>
       </c>
       <c r="D72">
-        <v>4100</v>
+        <v>10361.8</v>
       </c>
     </row>
     <row r="73">
@@ -3170,7 +3176,7 @@
         <v>Total</v>
       </c>
       <c r="D73">
-        <v>10361.8</v>
+        <v>5481</v>
       </c>
     </row>
     <row r="74">
@@ -3178,40 +3184,32 @@
         <v>Total</v>
       </c>
       <c r="D74">
-        <v>5481</v>
+        <v>3347.09</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D75">
-        <v>3347.09</v>
+        <v>📊  TOTAIS POR CATEGORIA</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>📊  TOTAIS POR CATEGORIA</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="str">
         <v>💰 TOTAL GERAL EMPRESA</v>
       </c>
-      <c r="D77">
+      <c r="D76">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H76"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:I104"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3841,13 +3839,16 @@
       </c>
     </row>
     <row r="38">
-      <c r="K38" t="str">
-        <v>🛑Atrasado</v>
+      <c r="A38" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="G39">
         <v>0</v>
@@ -3855,7 +3856,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Custos Variáveis</v>
+        <v>Impostos e Taxas</v>
       </c>
       <c r="G40">
         <v>0</v>
@@ -3863,7 +3864,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Impostos e Taxas</v>
+        <v>Pró-labore / Retirada</v>
       </c>
       <c r="G41">
         <v>0</v>
@@ -3871,10 +3872,31 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Pró-labore / Retirada</v>
+        <v>Agosto</v>
+      </c>
+      <c r="B42">
+        <v>46265</v>
+      </c>
+      <c r="C42">
+        <v>46265</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Estrutura</v>
       </c>
       <c r="G42">
-        <v>0</v>
+        <v>1000</v>
+      </c>
+      <c r="H42" t="str">
+        <v>✅ Pago</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Locação Estúdio / Espaço PJ</v>
       </c>
     </row>
     <row r="43">
@@ -3882,28 +3904,28 @@
         <v>Agosto</v>
       </c>
       <c r="B43">
-        <v>46265</v>
+        <v>46244</v>
       </c>
       <c r="C43">
-        <v>46265</v>
+        <v>46244</v>
       </c>
       <c r="D43" t="str">
-        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
+        <v>Google On</v>
       </c>
       <c r="E43" t="str">
         <v>Custos Fixos</v>
       </c>
       <c r="F43" t="str">
-        <v>Estrutura</v>
+        <v>Softwares</v>
       </c>
       <c r="G43">
-        <v>1000</v>
+        <v>96.99</v>
       </c>
       <c r="H43" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I43" t="str">
-        <v>Locação Estúdio / Espaço PJ</v>
+        <v>Armazenamento Nuvem</v>
       </c>
     </row>
     <row r="44">
@@ -3911,13 +3933,13 @@
         <v>Agosto</v>
       </c>
       <c r="B44">
-        <v>46244</v>
+        <v>46254</v>
       </c>
       <c r="C44">
-        <v>46244</v>
+        <v>46254</v>
       </c>
       <c r="D44" t="str">
-        <v>Google On</v>
+        <v>Adobe Creative Cloud</v>
       </c>
       <c r="E44" t="str">
         <v>Custos Fixos</v>
@@ -3926,13 +3948,13 @@
         <v>Softwares</v>
       </c>
       <c r="G44">
-        <v>96.99</v>
+        <v>129</v>
       </c>
       <c r="H44" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I44" t="str">
-        <v>Armazenamento Nuvem</v>
+        <v>Plano Aplicativos Adobe</v>
       </c>
     </row>
     <row r="45">
@@ -3940,28 +3962,28 @@
         <v>Agosto</v>
       </c>
       <c r="B45">
-        <v>46254</v>
+        <v>46252</v>
       </c>
       <c r="C45">
-        <v>46254</v>
+        <v>46252</v>
       </c>
       <c r="D45" t="str">
-        <v>Adobe Creative Cloud</v>
+        <v>Contador / Honorários - Isabel Almeida</v>
       </c>
       <c r="E45" t="str">
         <v>Custos Fixos</v>
       </c>
       <c r="F45" t="str">
-        <v>Softwares</v>
+        <v>Contabilidade</v>
       </c>
       <c r="G45">
-        <v>129</v>
+        <v>250</v>
       </c>
       <c r="H45" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I45" t="str">
-        <v>Plano Aplicativos Adobe</v>
+        <v>Honorários Contábeis PJ</v>
       </c>
     </row>
     <row r="46">
@@ -3969,28 +3991,28 @@
         <v>Agosto</v>
       </c>
       <c r="B46">
-        <v>46252</v>
+        <v>46256</v>
       </c>
       <c r="C46">
-        <v>46252</v>
+        <v>46256</v>
       </c>
       <c r="D46" t="str">
-        <v>Contador / Honorários - Isabel Almeida</v>
+        <v>Contador / Consultoria - Isabel Almeida</v>
       </c>
       <c r="E46" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F46" t="str">
         <v>Contabilidade</v>
       </c>
       <c r="G46">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="H46" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I46" t="str">
-        <v>Honorários Contábeis PJ</v>
+        <v>Serviços / Consultoria Contábil</v>
       </c>
     </row>
     <row r="47">
@@ -3998,28 +4020,28 @@
         <v>Agosto</v>
       </c>
       <c r="B47">
-        <v>46256</v>
+        <v>46247</v>
       </c>
       <c r="C47">
-        <v>46256</v>
+        <v>46247</v>
       </c>
       <c r="D47" t="str">
-        <v>Contador / Consultoria - Isabel Almeida</v>
+        <v>Equipe Vídeo/Foto - Marcelo Alves</v>
       </c>
       <c r="E47" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F47" t="str">
-        <v>Contabilidade</v>
+        <v>Equipe / Terceiros</v>
       </c>
       <c r="G47">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="H47" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I47" t="str">
-        <v>Serviços / Consultoria Contábil</v>
+        <v>Gabi Nutri - Cobertura Vídeo</v>
       </c>
     </row>
     <row r="48">
@@ -4027,10 +4049,10 @@
         <v>Agosto</v>
       </c>
       <c r="B48">
-        <v>46247</v>
+        <v>46261</v>
       </c>
       <c r="C48">
-        <v>46247</v>
+        <v>46261</v>
       </c>
       <c r="D48" t="str">
         <v>Equipe Vídeo/Foto - Marcelo Alves</v>
@@ -4048,7 +4070,7 @@
         <v>✅ Pago</v>
       </c>
       <c r="I48" t="str">
-        <v>Gabi Nutri - Cobertura Vídeo</v>
+        <v>Winner RH - Cobertura Vídeo</v>
       </c>
     </row>
     <row r="49">
@@ -4056,28 +4078,28 @@
         <v>Agosto</v>
       </c>
       <c r="B49">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="C49">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="D49" t="str">
-        <v>Equipe Vídeo/Foto - Marcelo Alves</v>
+        <v>Apoio Operacional - Andrea Fernandes</v>
       </c>
       <c r="E49" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F49" t="str">
-        <v>Equipe / Terceiros</v>
+        <v>Equipe / Apoio</v>
       </c>
       <c r="G49">
-        <v>800</v>
+        <v>250</v>
       </c>
       <c r="H49" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I49" t="str">
-        <v>Winner RH - Cobertura Vídeo</v>
+        <v>Apoio Operacional 1/2</v>
       </c>
     </row>
     <row r="50">
@@ -4085,10 +4107,10 @@
         <v>Agosto</v>
       </c>
       <c r="B50">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="C50">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="D50" t="str">
         <v>Apoio Operacional - Andrea Fernandes</v>
@@ -4100,13 +4122,13 @@
         <v>Equipe / Apoio</v>
       </c>
       <c r="G50">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="H50" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I50" t="str">
-        <v>Apoio Operacional 1/2</v>
+        <v>Apoio Operacional 2/2</v>
       </c>
     </row>
     <row r="51">
@@ -4114,28 +4136,28 @@
         <v>Agosto</v>
       </c>
       <c r="B51">
-        <v>46265</v>
+        <v>46253</v>
       </c>
       <c r="C51">
-        <v>46265</v>
+        <v>46253</v>
       </c>
       <c r="D51" t="str">
-        <v>Apoio Operacional - Andrea Fernandes</v>
+        <v>Taxas de Gateway - Pagar.me / Stone</v>
       </c>
       <c r="E51" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F51" t="str">
-        <v>Equipe / Apoio</v>
+        <v>Taxas Financeiras</v>
       </c>
       <c r="G51">
-        <v>50</v>
+        <v>182.2</v>
       </c>
       <c r="H51" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I51" t="str">
-        <v>Apoio Operacional 2/2</v>
+        <v>Taxas transacionais gateway</v>
       </c>
     </row>
     <row r="52">
@@ -4143,28 +4165,28 @@
         <v>Agosto</v>
       </c>
       <c r="B52">
-        <v>46253</v>
+        <v>46244</v>
       </c>
       <c r="C52">
-        <v>46253</v>
+        <v>46244</v>
       </c>
       <c r="D52" t="str">
-        <v>Taxas de Gateway - Pagar.me / Stone</v>
+        <v>Estacionamento / Produção - P L Moura</v>
       </c>
       <c r="E52" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F52" t="str">
-        <v>Taxas Financeiras</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G52">
-        <v>182.2</v>
+        <v>89.68</v>
       </c>
       <c r="H52" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I52" t="str">
-        <v>Taxas transacionais gateway</v>
+        <v>Estacionamentos em produções/reuniões</v>
       </c>
     </row>
     <row r="53">
@@ -4172,28 +4194,28 @@
         <v>Agosto</v>
       </c>
       <c r="B53">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="C53">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="D53" t="str">
-        <v>Estacionamento / Produção - P L Moura</v>
+        <v>Amazon Prime / Digital</v>
       </c>
       <c r="E53" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F53" t="str">
-        <v>Transporte / Produção</v>
+        <v>Serviços Digitais</v>
       </c>
       <c r="G53">
-        <v>89.68</v>
+        <v>54.8</v>
       </c>
       <c r="H53" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I53" t="str">
-        <v>Estacionamentos em produções/reuniões</v>
+        <v>29.90 + 24.90</v>
       </c>
     </row>
     <row r="54">
@@ -4201,28 +4223,28 @@
         <v>Agosto</v>
       </c>
       <c r="B54">
-        <v>46240</v>
+        <v>46254</v>
       </c>
       <c r="C54">
-        <v>46240</v>
+        <v>46254</v>
       </c>
       <c r="D54" t="str">
-        <v>Amazon Prime / Digital</v>
+        <v>Canva Pro</v>
       </c>
       <c r="E54" t="str">
         <v>Custos Fixos</v>
       </c>
       <c r="F54" t="str">
-        <v>Serviços Digitais</v>
+        <v>Softwares</v>
       </c>
       <c r="G54">
-        <v>54.8</v>
+        <v>47</v>
       </c>
       <c r="H54" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I54" t="str">
-        <v>29.90 + 24.90</v>
+        <v>Assinatura Canva (pago via NuPay PF)</v>
       </c>
     </row>
     <row r="55">
@@ -4230,28 +4252,28 @@
         <v>Agosto</v>
       </c>
       <c r="B55">
-        <v>46254</v>
+        <v>46260</v>
       </c>
       <c r="C55">
-        <v>46254</v>
+        <v>46260</v>
       </c>
       <c r="D55" t="str">
-        <v>Canva Pro</v>
+        <v>Meta Ads (Facebook Ads)</v>
       </c>
       <c r="E55" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F55" t="str">
-        <v>Softwares</v>
+        <v>Marketing / Ads</v>
       </c>
       <c r="G55">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H55" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I55" t="str">
-        <v>Assinatura Canva (pago via NuPay PF)</v>
+        <v>Anúncios Meta (pago via NuPay PF)</v>
       </c>
     </row>
     <row r="56">
@@ -4259,28 +4281,25 @@
         <v>Agosto</v>
       </c>
       <c r="B56">
-        <v>46260</v>
-      </c>
-      <c r="C56">
-        <v>46260</v>
+        <v>46264</v>
       </c>
       <c r="D56" t="str">
-        <v>Meta Ads (Facebook Ads)</v>
+        <v>DAS Simples Nacional</v>
       </c>
       <c r="E56" t="str">
-        <v>Custos Variáveis</v>
+        <v>Impostos e Taxas</v>
       </c>
       <c r="F56" t="str">
-        <v>Marketing / Ads</v>
+        <v>Impostos</v>
       </c>
       <c r="G56">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="H56" t="str">
-        <v>✅ Pago</v>
+        <v>⏳ Pendente</v>
       </c>
       <c r="I56" t="str">
-        <v>Anúncios Meta (pago via NuPay PF)</v>
+        <v>Aguardando apuração da contabilidade</v>
       </c>
     </row>
     <row r="57">
@@ -4288,51 +4307,54 @@
         <v>Agosto</v>
       </c>
       <c r="B57">
-        <v>46264</v>
+        <v>46263</v>
       </c>
       <c r="D57" t="str">
-        <v>DAS Simples Nacional</v>
+        <v>Renegociação PJ</v>
       </c>
       <c r="E57" t="str">
-        <v>Impostos e Taxas</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F57" t="str">
-        <v>Impostos</v>
+        <v>Dívidas PJ</v>
       </c>
       <c r="G57">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="H57" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="I57" t="str">
-        <v>Aguardando apuração da contabilidade</v>
+        <v>Parcelamento PJ</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Agosto</v>
+        <v>Junho</v>
       </c>
       <c r="B58">
-        <v>46263</v>
+        <v>46174</v>
+      </c>
+      <c r="C58">
+        <v>46174</v>
       </c>
       <c r="D58" t="str">
-        <v>Renegociação PJ</v>
+        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
       </c>
       <c r="E58" t="str">
         <v>Custos Fixos</v>
       </c>
       <c r="F58" t="str">
-        <v>Dívidas PJ</v>
+        <v>Estrutura</v>
       </c>
       <c r="G58">
-        <v>60</v>
+        <v>1000</v>
       </c>
       <c r="H58" t="str">
-        <v>⏳ Pendente</v>
+        <v>✅ Pago</v>
       </c>
       <c r="I58" t="str">
-        <v>Parcelamento PJ</v>
+        <v>Locação Estúdio / Espaço PJ</v>
       </c>
     </row>
     <row r="59">
@@ -4340,28 +4362,28 @@
         <v>Junho</v>
       </c>
       <c r="B59">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="C59">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="D59" t="str">
-        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
+        <v>Estacionamento / Produção (P L Moura)</v>
       </c>
       <c r="E59" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F59" t="str">
-        <v>Estrutura</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G59">
-        <v>1000</v>
+        <v>30.89</v>
       </c>
       <c r="H59" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I59" t="str">
-        <v>Locação Estúdio / Espaço PJ</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="60">
@@ -4369,28 +4391,28 @@
         <v>Junho</v>
       </c>
       <c r="B60">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="C60">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="D60" t="str">
-        <v>Estacionamento / Produção (P L Moura)</v>
+        <v>Contador / Honorários (Marenn)</v>
       </c>
       <c r="E60" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F60" t="str">
-        <v>Transporte / Produção</v>
+        <v>Contabilidade</v>
       </c>
       <c r="G60">
-        <v>30.89</v>
+        <v>55.21</v>
       </c>
       <c r="H60" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I60" t="str">
-        <v>Estacionamento</v>
+        <v>Honorários Contábeis</v>
       </c>
     </row>
     <row r="61">
@@ -4404,22 +4426,22 @@
         <v>46176</v>
       </c>
       <c r="D61" t="str">
-        <v>Contador / Honorários (Marenn)</v>
+        <v>Taxas de Gateway (Pagar.me)</v>
       </c>
       <c r="E61" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F61" t="str">
-        <v>Contabilidade</v>
+        <v>Taxas Financeiras</v>
       </c>
       <c r="G61">
-        <v>55.21</v>
+        <v>62.28</v>
       </c>
       <c r="H61" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I61" t="str">
-        <v>Honorários Contábeis</v>
+        <v>Taxas transacionais</v>
       </c>
     </row>
     <row r="62">
@@ -4427,28 +4449,28 @@
         <v>Junho</v>
       </c>
       <c r="B62">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="C62">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="D62" t="str">
-        <v>Taxas de Gateway (Pagar.me)</v>
+        <v>Equipe / Serviços (Sergio Xavier)</v>
       </c>
       <c r="E62" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F62" t="str">
-        <v>Taxas Financeiras</v>
+        <v>Equipe / Terceiros</v>
       </c>
       <c r="G62">
-        <v>62.28</v>
+        <v>190</v>
       </c>
       <c r="H62" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I62" t="str">
-        <v>Taxas transacionais</v>
+        <v>Produção Audiovisual</v>
       </c>
     </row>
     <row r="63">
@@ -4456,28 +4478,28 @@
         <v>Junho</v>
       </c>
       <c r="B63">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="C63">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="D63" t="str">
-        <v>Equipe / Serviços (Sergio Xavier)</v>
+        <v>Estacionamento (Brasil Park)</v>
       </c>
       <c r="E63" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F63" t="str">
-        <v>Equipe / Terceiros</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G63">
-        <v>190</v>
+        <v>24</v>
       </c>
       <c r="H63" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I63" t="str">
-        <v>Produção Audiovisual</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="64">
@@ -4491,22 +4513,22 @@
         <v>46178</v>
       </c>
       <c r="D64" t="str">
-        <v>Estacionamento (Brasil Park)</v>
+        <v>Despesa Operacional (M4 Produtos)</v>
       </c>
       <c r="E64" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F64" t="str">
-        <v>Transporte / Produção</v>
+        <v>Operacional</v>
       </c>
       <c r="G64">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H64" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I64" t="str">
-        <v>Estacionamento</v>
+        <v>Insumos PJ</v>
       </c>
     </row>
     <row r="65">
@@ -4514,28 +4536,28 @@
         <v>Junho</v>
       </c>
       <c r="B65">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="C65">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="D65" t="str">
-        <v>Despesa Operacional (M4 Produtos)</v>
+        <v>Estacionamento / Produção (P L Moura)</v>
       </c>
       <c r="E65" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F65" t="str">
-        <v>Operacional</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G65">
-        <v>25</v>
+        <v>18.9</v>
       </c>
       <c r="H65" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I65" t="str">
-        <v>Insumos PJ</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="66">
@@ -4543,28 +4565,28 @@
         <v>Junho</v>
       </c>
       <c r="B66">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="C66">
-        <v>46179</v>
+        <v>46180</v>
       </c>
       <c r="D66" t="str">
-        <v>Estacionamento / Produção (P L Moura)</v>
+        <v>Apoio / Serviços (Janaina Duarte)</v>
       </c>
       <c r="E66" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F66" t="str">
-        <v>Transporte / Produção</v>
+        <v>Equipe / Apoio</v>
       </c>
       <c r="G66">
-        <v>18.9</v>
+        <v>50</v>
       </c>
       <c r="H66" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I66" t="str">
-        <v>Estacionamento</v>
+        <v>Serviços Apoio</v>
       </c>
     </row>
     <row r="67">
@@ -4572,28 +4594,28 @@
         <v>Junho</v>
       </c>
       <c r="B67">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="C67">
-        <v>46180</v>
+        <v>46181</v>
       </c>
       <c r="D67" t="str">
-        <v>Apoio / Serviços (Janaina Duarte)</v>
+        <v>Estacionamento / Produção (P L Moura)</v>
       </c>
       <c r="E67" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F67" t="str">
-        <v>Equipe / Apoio</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G67">
-        <v>50</v>
+        <v>18.9</v>
       </c>
       <c r="H67" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I67" t="str">
-        <v>Serviços Apoio</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="68">
@@ -4601,28 +4623,28 @@
         <v>Junho</v>
       </c>
       <c r="B68">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="C68">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="D68" t="str">
-        <v>Estacionamento / Produção (P L Moura)</v>
+        <v>Meta Ads (Facebook Ads)</v>
       </c>
       <c r="E68" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F68" t="str">
-        <v>Transporte / Produção</v>
+        <v>Marketing / Ads</v>
       </c>
       <c r="G68">
-        <v>18.9</v>
+        <v>136.69</v>
       </c>
       <c r="H68" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I68" t="str">
-        <v>Estacionamento</v>
+        <v>Anúncios Meta Ads</v>
       </c>
     </row>
     <row r="69">
@@ -4630,28 +4652,28 @@
         <v>Junho</v>
       </c>
       <c r="B69">
-        <v>46182</v>
+        <v>46187</v>
       </c>
       <c r="C69">
-        <v>46182</v>
+        <v>46187</v>
       </c>
       <c r="D69" t="str">
-        <v>Meta Ads (Facebook Ads)</v>
+        <v>Equipe / Edição (Rafael Martins)</v>
       </c>
       <c r="E69" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F69" t="str">
-        <v>Marketing / Ads</v>
+        <v>Equipe / Terceiros</v>
       </c>
       <c r="G69">
-        <v>136.69</v>
+        <v>1000</v>
       </c>
       <c r="H69" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I69" t="str">
-        <v>Anúncios Meta Ads</v>
+        <v>Edição / Produção Vídeo</v>
       </c>
     </row>
     <row r="70">
@@ -4659,28 +4681,28 @@
         <v>Junho</v>
       </c>
       <c r="B70">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="C70">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="D70" t="str">
-        <v>Equipe / Edição (Rafael Martins)</v>
+        <v>Sistemas / Software (Intelisoft)</v>
       </c>
       <c r="E70" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F70" t="str">
-        <v>Equipe / Terceiros</v>
+        <v>Softwares</v>
       </c>
       <c r="G70">
-        <v>1000</v>
+        <v>59.9</v>
       </c>
       <c r="H70" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I70" t="str">
-        <v>Edição / Produção Vídeo</v>
+        <v>Sistema</v>
       </c>
     </row>
     <row r="71">
@@ -4694,22 +4716,22 @@
         <v>46188</v>
       </c>
       <c r="D71" t="str">
-        <v>Sistemas / Software (Intelisoft)</v>
+        <v>Contador / Honorários (Marenn)</v>
       </c>
       <c r="E71" t="str">
         <v>Custos Fixos</v>
       </c>
       <c r="F71" t="str">
-        <v>Softwares</v>
+        <v>Contabilidade</v>
       </c>
       <c r="G71">
-        <v>59.9</v>
+        <v>70.77</v>
       </c>
       <c r="H71" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I71" t="str">
-        <v>Sistema</v>
+        <v>Honorários Contábeis</v>
       </c>
     </row>
     <row r="72">
@@ -4717,28 +4739,28 @@
         <v>Junho</v>
       </c>
       <c r="B72">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="C72">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="D72" t="str">
-        <v>Contador / Honorários (Marenn)</v>
+        <v>Estacionamento / Produção (P L Moura)</v>
       </c>
       <c r="E72" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F72" t="str">
-        <v>Contabilidade</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G72">
-        <v>70.77</v>
+        <v>18.9</v>
       </c>
       <c r="H72" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I72" t="str">
-        <v>Honorários Contábeis</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="73">
@@ -4746,10 +4768,10 @@
         <v>Junho</v>
       </c>
       <c r="B73">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="C73">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="D73" t="str">
         <v>Estacionamento / Produção (P L Moura)</v>
@@ -4781,22 +4803,22 @@
         <v>46190</v>
       </c>
       <c r="D74" t="str">
-        <v>Estacionamento / Produção (P L Moura)</v>
+        <v>Meta Ads (Facebook Ads)</v>
       </c>
       <c r="E74" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F74" t="str">
-        <v>Transporte / Produção</v>
+        <v>Marketing / Ads</v>
       </c>
       <c r="G74">
-        <v>18.9</v>
+        <v>103</v>
       </c>
       <c r="H74" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I74" t="str">
-        <v>Estacionamento</v>
+        <v>Anúncios Meta Ads</v>
       </c>
     </row>
     <row r="75">
@@ -4804,10 +4826,10 @@
         <v>Junho</v>
       </c>
       <c r="B75">
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="C75">
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="D75" t="str">
         <v>Meta Ads (Facebook Ads)</v>
@@ -4819,7 +4841,7 @@
         <v>Marketing / Ads</v>
       </c>
       <c r="G75">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H75" t="str">
         <v>✅ Pago</v>
@@ -4833,28 +4855,28 @@
         <v>Junho</v>
       </c>
       <c r="B76">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="C76">
-        <v>46192</v>
+        <v>46193</v>
       </c>
       <c r="D76" t="str">
-        <v>Meta Ads (Facebook Ads)</v>
+        <v>Tarifas Bancárias (Débito Conta)</v>
       </c>
       <c r="E76" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F76" t="str">
-        <v>Marketing / Ads</v>
+        <v>Taxas Bancárias</v>
       </c>
       <c r="G76">
-        <v>100</v>
+        <v>32.9</v>
       </c>
       <c r="H76" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I76" t="str">
-        <v>Anúncios Meta Ads</v>
+        <v>Tarifa de Conta PJ</v>
       </c>
     </row>
     <row r="77">
@@ -4868,22 +4890,22 @@
         <v>46193</v>
       </c>
       <c r="D77" t="str">
-        <v>Tarifas Bancárias (Débito Conta)</v>
+        <v>Estacionamento (Unita Park)</v>
       </c>
       <c r="E77" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F77" t="str">
-        <v>Taxas Bancárias</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G77">
-        <v>32.9</v>
+        <v>23</v>
       </c>
       <c r="H77" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I77" t="str">
-        <v>Tarifa de Conta PJ</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="78">
@@ -4897,22 +4919,22 @@
         <v>46193</v>
       </c>
       <c r="D78" t="str">
-        <v>Estacionamento (Unita Park)</v>
+        <v>Equipe / Apoio (Tatiana Gonçalves)</v>
       </c>
       <c r="E78" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F78" t="str">
-        <v>Transporte / Produção</v>
+        <v>Equipe / Apoio</v>
       </c>
       <c r="G78">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="H78" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I78" t="str">
-        <v>Estacionamento</v>
+        <v>Apoio Produção</v>
       </c>
     </row>
     <row r="79">
@@ -4920,28 +4942,28 @@
         <v>Junho</v>
       </c>
       <c r="B79">
-        <v>46193</v>
+        <v>46196</v>
       </c>
       <c r="C79">
-        <v>46193</v>
+        <v>46196</v>
       </c>
       <c r="D79" t="str">
-        <v>Equipe / Apoio (Tatiana Gonçalves)</v>
+        <v>Aluguel do Estúdio - Complemento (Julio Cesar)</v>
       </c>
       <c r="E79" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F79" t="str">
-        <v>Equipe / Apoio</v>
+        <v>Estrutura</v>
       </c>
       <c r="G79">
-        <v>150</v>
+        <v>900</v>
       </c>
       <c r="H79" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I79" t="str">
-        <v>Apoio Produção</v>
+        <v>Aluguel Estúdio</v>
       </c>
     </row>
     <row r="80">
@@ -4955,22 +4977,22 @@
         <v>46196</v>
       </c>
       <c r="D80" t="str">
-        <v>Aluguel do Estúdio - Complemento (Julio Cesar)</v>
+        <v>Estacionamento / Produção (P L Moura)</v>
       </c>
       <c r="E80" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F80" t="str">
-        <v>Estrutura</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G80">
-        <v>900</v>
+        <v>11.8</v>
       </c>
       <c r="H80" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I80" t="str">
-        <v>Aluguel Estúdio</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="81">
@@ -4978,28 +5000,28 @@
         <v>Junho</v>
       </c>
       <c r="B81">
-        <v>46196</v>
+        <v>46199</v>
       </c>
       <c r="C81">
-        <v>46196</v>
+        <v>46199</v>
       </c>
       <c r="D81" t="str">
-        <v>Estacionamento / Produção (P L Moura)</v>
+        <v>Apoio / Serviços (Grazielle Silva)</v>
       </c>
       <c r="E81" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F81" t="str">
-        <v>Transporte / Produção</v>
+        <v>Equipe / Apoio</v>
       </c>
       <c r="G81">
-        <v>11.8</v>
+        <v>100</v>
       </c>
       <c r="H81" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I81" t="str">
-        <v>Estacionamento</v>
+        <v>Serviços Apoio</v>
       </c>
     </row>
     <row r="82">
@@ -5007,19 +5029,19 @@
         <v>Junho</v>
       </c>
       <c r="B82">
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="C82">
-        <v>46199</v>
+        <v>46202</v>
       </c>
       <c r="D82" t="str">
-        <v>Apoio / Serviços (Grazielle Silva)</v>
+        <v>Aluguel do Estúdio - Complemento (Julio Cesar)</v>
       </c>
       <c r="E82" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F82" t="str">
-        <v>Equipe / Apoio</v>
+        <v>Estrutura</v>
       </c>
       <c r="G82">
         <v>100</v>
@@ -5028,36 +5050,36 @@
         <v>✅ Pago</v>
       </c>
       <c r="I82" t="str">
-        <v>Serviços Apoio</v>
+        <v>Aluguel Estúdio</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Junho</v>
+        <v>Julho</v>
       </c>
       <c r="B83">
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="C83">
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="D83" t="str">
-        <v>Aluguel do Estúdio - Complemento (Julio Cesar)</v>
+        <v>Equipe / Apoio (Tatiana Gonçalves)</v>
       </c>
       <c r="E83" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F83" t="str">
-        <v>Estrutura</v>
+        <v>Equipe / Apoio</v>
       </c>
       <c r="G83">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H83" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I83" t="str">
-        <v>Aluguel Estúdio</v>
+        <v>Apoio Produção 1/2</v>
       </c>
     </row>
     <row r="84">
@@ -5065,10 +5087,10 @@
         <v>Julho</v>
       </c>
       <c r="B84">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="C84">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="D84" t="str">
         <v>Equipe / Apoio (Tatiana Gonçalves)</v>
@@ -5080,13 +5102,13 @@
         <v>Equipe / Apoio</v>
       </c>
       <c r="G84">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="H84" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I84" t="str">
-        <v>Apoio Produção 1/2</v>
+        <v>Apoio Produção 2/2</v>
       </c>
     </row>
     <row r="85">
@@ -5094,28 +5116,28 @@
         <v>Julho</v>
       </c>
       <c r="B85">
-        <v>46206</v>
+        <v>46208</v>
       </c>
       <c r="C85">
-        <v>46206</v>
+        <v>46208</v>
       </c>
       <c r="D85" t="str">
-        <v>Equipe / Apoio (Tatiana Gonçalves)</v>
+        <v>Meta Ads (Facebook Ads)</v>
       </c>
       <c r="E85" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F85" t="str">
-        <v>Equipe / Apoio</v>
+        <v>Marketing / Ads</v>
       </c>
       <c r="G85">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="H85" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I85" t="str">
-        <v>Apoio Produção 2/2</v>
+        <v>Anúncios Meta Ads</v>
       </c>
     </row>
     <row r="86">
@@ -5129,22 +5151,22 @@
         <v>46208</v>
       </c>
       <c r="D86" t="str">
-        <v>Meta Ads (Facebook Ads)</v>
+        <v>Manutenção Estúdio (Amoedo Recreio)</v>
       </c>
       <c r="E86" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F86" t="str">
-        <v>Marketing / Ads</v>
+        <v>Estrutura</v>
       </c>
       <c r="G86">
-        <v>150</v>
+        <v>21.9</v>
       </c>
       <c r="H86" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I86" t="str">
-        <v>Anúncios Meta Ads</v>
+        <v>Insumos Estúdio</v>
       </c>
     </row>
     <row r="87">
@@ -5158,22 +5180,22 @@
         <v>46208</v>
       </c>
       <c r="D87" t="str">
-        <v>Manutenção Estúdio (Amoedo Recreio)</v>
+        <v>Estacionamento / Produção (P L Moura)</v>
       </c>
       <c r="E87" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F87" t="str">
-        <v>Estrutura</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G87">
-        <v>21.9</v>
+        <v>11.8</v>
       </c>
       <c r="H87" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I87" t="str">
-        <v>Insumos Estúdio</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="88">
@@ -5181,10 +5203,10 @@
         <v>Julho</v>
       </c>
       <c r="B88">
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="C88">
-        <v>46208</v>
+        <v>46211</v>
       </c>
       <c r="D88" t="str">
         <v>Estacionamento / Produção (P L Moura)</v>
@@ -5210,28 +5232,28 @@
         <v>Julho</v>
       </c>
       <c r="B89">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="C89">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="D89" t="str">
-        <v>Estacionamento / Produção (P L Moura)</v>
+        <v>Contador / Honorários (Isabel Almeida)</v>
       </c>
       <c r="E89" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F89" t="str">
-        <v>Transporte / Produção</v>
+        <v>Contabilidade</v>
       </c>
       <c r="G89">
-        <v>11.8</v>
+        <v>400</v>
       </c>
       <c r="H89" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I89" t="str">
-        <v>Estacionamento</v>
+        <v>Honorários Contábeis PJ</v>
       </c>
     </row>
     <row r="90">
@@ -5239,28 +5261,28 @@
         <v>Julho</v>
       </c>
       <c r="B90">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="C90">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="D90" t="str">
-        <v>Contador / Honorários (Isabel Almeida)</v>
+        <v>Meta Ads (Facebook Ads)</v>
       </c>
       <c r="E90" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F90" t="str">
-        <v>Contabilidade</v>
+        <v>Marketing / Ads</v>
       </c>
       <c r="G90">
-        <v>400</v>
+        <v>102</v>
       </c>
       <c r="H90" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I90" t="str">
-        <v>Honorários Contábeis PJ</v>
+        <v>Anúncios Meta Ads</v>
       </c>
     </row>
     <row r="91">
@@ -5268,28 +5290,28 @@
         <v>Julho</v>
       </c>
       <c r="B91">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="C91">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="D91" t="str">
-        <v>Meta Ads (Facebook Ads)</v>
+        <v>Estacionamento / Produção (P L Moura)</v>
       </c>
       <c r="E91" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F91" t="str">
-        <v>Marketing / Ads</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G91">
-        <v>102</v>
+        <v>11.8</v>
       </c>
       <c r="H91" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I91" t="str">
-        <v>Anúncios Meta Ads</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="92">
@@ -5297,28 +5319,28 @@
         <v>Julho</v>
       </c>
       <c r="B92">
-        <v>46217</v>
+        <v>46223</v>
       </c>
       <c r="C92">
-        <v>46217</v>
+        <v>46223</v>
       </c>
       <c r="D92" t="str">
-        <v>Estacionamento / Produção (P L Moura)</v>
+        <v>Tarifas Bancárias (Débito Conta)</v>
       </c>
       <c r="E92" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F92" t="str">
-        <v>Transporte / Produção</v>
+        <v>Taxas Bancárias</v>
       </c>
       <c r="G92">
-        <v>11.8</v>
+        <v>32.9</v>
       </c>
       <c r="H92" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I92" t="str">
-        <v>Estacionamento</v>
+        <v>Tarifa de Conta PJ</v>
       </c>
     </row>
     <row r="93">
@@ -5332,22 +5354,22 @@
         <v>46223</v>
       </c>
       <c r="D93" t="str">
-        <v>Tarifas Bancárias (Débito Conta)</v>
+        <v>Canva Pro</v>
       </c>
       <c r="E93" t="str">
         <v>Custos Fixos</v>
       </c>
       <c r="F93" t="str">
-        <v>Taxas Bancárias</v>
+        <v>Softwares</v>
       </c>
       <c r="G93">
-        <v>32.9</v>
+        <v>47</v>
       </c>
       <c r="H93" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I93" t="str">
-        <v>Tarifa de Conta PJ</v>
+        <v>Assinatura Canva (via PF)</v>
       </c>
     </row>
     <row r="94">
@@ -5355,28 +5377,28 @@
         <v>Julho</v>
       </c>
       <c r="B94">
-        <v>46223</v>
+        <v>46227</v>
       </c>
       <c r="C94">
-        <v>46223</v>
+        <v>46227</v>
       </c>
       <c r="D94" t="str">
-        <v>Canva Pro</v>
+        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
       </c>
       <c r="E94" t="str">
         <v>Custos Fixos</v>
       </c>
       <c r="F94" t="str">
-        <v>Softwares</v>
+        <v>Estrutura</v>
       </c>
       <c r="G94">
-        <v>47</v>
+        <v>800</v>
       </c>
       <c r="H94" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I94" t="str">
-        <v>Assinatura Canva (via PF)</v>
+        <v>Locação Estúdio / Espaço PJ</v>
       </c>
     </row>
     <row r="95">
@@ -5384,28 +5406,28 @@
         <v>Julho</v>
       </c>
       <c r="B95">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="C95">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="D95" t="str">
-        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
+        <v>Estacionamento / Produção (P L Moura)</v>
       </c>
       <c r="E95" t="str">
-        <v>Custos Fixos</v>
+        <v>Custos Variáveis</v>
       </c>
       <c r="F95" t="str">
-        <v>Estrutura</v>
+        <v>Transporte / Produção</v>
       </c>
       <c r="G95">
-        <v>800</v>
+        <v>11.8</v>
       </c>
       <c r="H95" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I95" t="str">
-        <v>Locação Estúdio / Espaço PJ</v>
+        <v>Estacionamento</v>
       </c>
     </row>
     <row r="96">
@@ -5419,22 +5441,22 @@
         <v>46231</v>
       </c>
       <c r="D96" t="str">
-        <v>Estacionamento / Produção (P L Moura)</v>
+        <v>Equipe / Produção (Thiago Santa Martha)</v>
       </c>
       <c r="E96" t="str">
         <v>Custos Variáveis</v>
       </c>
       <c r="F96" t="str">
-        <v>Transporte / Produção</v>
+        <v>Equipe / Terceiros</v>
       </c>
       <c r="G96">
-        <v>11.8</v>
+        <v>1000</v>
       </c>
       <c r="H96" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I96" t="str">
-        <v>Estacionamento</v>
+        <v>Produção Audiovisual</v>
       </c>
     </row>
     <row r="97">
@@ -5442,57 +5464,36 @@
         <v>Julho</v>
       </c>
       <c r="B97">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C97">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="D97" t="str">
-        <v>Equipe / Produção (Thiago Santa Martha)</v>
+        <v>Aluguel do Estúdio - Complemento (Julio Cesar)</v>
       </c>
       <c r="E97" t="str">
-        <v>Custos Variáveis</v>
+        <v>Custos Fixos</v>
       </c>
       <c r="F97" t="str">
-        <v>Equipe / Terceiros</v>
+        <v>Estrutura</v>
       </c>
       <c r="G97">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="H97" t="str">
         <v>✅ Pago</v>
       </c>
       <c r="I97" t="str">
-        <v>Produção Audiovisual</v>
+        <v>Aluguel Estúdio</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Julho</v>
-      </c>
-      <c r="B98">
-        <v>46232</v>
-      </c>
-      <c r="C98">
-        <v>46232</v>
-      </c>
-      <c r="D98" t="str">
-        <v>Aluguel do Estúdio - Complemento (Julio Cesar)</v>
-      </c>
-      <c r="E98" t="str">
-        <v>Custos Fixos</v>
-      </c>
-      <c r="F98" t="str">
-        <v>Estrutura</v>
-      </c>
-      <c r="G98">
-        <v>200</v>
-      </c>
-      <c r="H98" t="str">
-        <v>✅ Pago</v>
-      </c>
-      <c r="I98" t="str">
-        <v>Aluguel Estúdio</v>
+        <v>Total</v>
+      </c>
+      <c r="D98">
+        <v>2638.54</v>
       </c>
     </row>
     <row r="99">
@@ -5500,7 +5501,7 @@
         <v>Total</v>
       </c>
       <c r="D99">
-        <v>2638.54</v>
+        <v>2111.89</v>
       </c>
     </row>
     <row r="100">
@@ -5508,7 +5509,7 @@
         <v>Total</v>
       </c>
       <c r="D100">
-        <v>2111.89</v>
+        <v>1751.89</v>
       </c>
     </row>
     <row r="101">
@@ -5524,33 +5525,25 @@
         <v>Total</v>
       </c>
       <c r="D102">
-        <v>1751.89</v>
+        <v>3601.89</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D103">
-        <v>3601.89</v>
+        <v>📊  TOTAIS POR CATEGORIA</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>📊  TOTAIS POR CATEGORIA</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="str">
         <v>💰 TOTAL GERAL EMPRESA</v>
       </c>
-      <c r="G105">
+      <c r="G104">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I104"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6346,6 +6339,9 @@
       </c>
     </row>
     <row r="47">
+      <c r="A47" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C47">
         <v>46123</v>
       </c>
@@ -6363,6 +6359,9 @@
       </c>
     </row>
     <row r="48">
+      <c r="A48" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C48">
         <v>46123</v>
       </c>
@@ -6380,6 +6379,9 @@
       </c>
     </row>
     <row r="49">
+      <c r="A49" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C49">
         <v>46123</v>
       </c>
@@ -6397,6 +6399,9 @@
       </c>
     </row>
     <row r="50">
+      <c r="A50" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C50">
         <v>46123</v>
       </c>
@@ -6414,6 +6419,9 @@
       </c>
     </row>
     <row r="51">
+      <c r="A51" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C51">
         <v>46123</v>
       </c>
@@ -6431,6 +6439,9 @@
       </c>
     </row>
     <row r="52">
+      <c r="A52" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C52">
         <v>46123</v>
       </c>
@@ -6448,6 +6459,9 @@
       </c>
     </row>
     <row r="53">
+      <c r="A53" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C53">
         <v>46124</v>
       </c>
@@ -6465,6 +6479,9 @@
       </c>
     </row>
     <row r="54">
+      <c r="A54" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C54">
         <v>46125</v>
       </c>
@@ -6482,6 +6499,9 @@
       </c>
     </row>
     <row r="55">
+      <c r="A55" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C55">
         <v>46125</v>
       </c>
@@ -6499,6 +6519,9 @@
       </c>
     </row>
     <row r="56">
+      <c r="A56" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C56">
         <v>46125</v>
       </c>
@@ -6516,6 +6539,9 @@
       </c>
     </row>
     <row r="57">
+      <c r="A57" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C57">
         <v>46125</v>
       </c>
@@ -6533,6 +6559,9 @@
       </c>
     </row>
     <row r="58">
+      <c r="A58" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C58">
         <v>46125</v>
       </c>
@@ -6550,6 +6579,9 @@
       </c>
     </row>
     <row r="59">
+      <c r="A59" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C59">
         <v>46126</v>
       </c>
@@ -6567,6 +6599,9 @@
       </c>
     </row>
     <row r="60">
+      <c r="A60" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C60">
         <v>46126</v>
       </c>
@@ -6584,6 +6619,9 @@
       </c>
     </row>
     <row r="61">
+      <c r="A61" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C61">
         <v>46126</v>
       </c>
@@ -6601,6 +6639,9 @@
       </c>
     </row>
     <row r="62">
+      <c r="A62" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C62">
         <v>46126</v>
       </c>
@@ -6618,6 +6659,9 @@
       </c>
     </row>
     <row r="63">
+      <c r="A63" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C63">
         <v>46127</v>
       </c>
@@ -6635,6 +6679,9 @@
       </c>
     </row>
     <row r="64">
+      <c r="A64" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C64">
         <v>46127</v>
       </c>
@@ -6652,6 +6699,9 @@
       </c>
     </row>
     <row r="65">
+      <c r="A65" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C65">
         <v>46127</v>
       </c>
@@ -6669,6 +6719,9 @@
       </c>
     </row>
     <row r="66">
+      <c r="A66" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C66">
         <v>46127</v>
       </c>
@@ -6686,6 +6739,9 @@
       </c>
     </row>
     <row r="67">
+      <c r="A67" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C67">
         <v>46128</v>
       </c>
@@ -6703,6 +6759,9 @@
       </c>
     </row>
     <row r="68">
+      <c r="A68" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C68">
         <v>46128</v>
       </c>
@@ -6720,6 +6779,9 @@
       </c>
     </row>
     <row r="69">
+      <c r="A69" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C69">
         <v>46128</v>
       </c>
@@ -6737,6 +6799,9 @@
       </c>
     </row>
     <row r="70">
+      <c r="A70" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C70">
         <v>46130</v>
       </c>
@@ -6754,6 +6819,9 @@
       </c>
     </row>
     <row r="71">
+      <c r="A71" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C71">
         <v>46131</v>
       </c>
@@ -6771,6 +6839,9 @@
       </c>
     </row>
     <row r="72">
+      <c r="A72" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C72">
         <v>46131</v>
       </c>
@@ -6788,6 +6859,9 @@
       </c>
     </row>
     <row r="73">
+      <c r="A73" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C73">
         <v>46131</v>
       </c>
@@ -6805,6 +6879,9 @@
       </c>
     </row>
     <row r="74">
+      <c r="A74" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C74">
         <v>46132</v>
       </c>
@@ -6822,6 +6899,9 @@
       </c>
     </row>
     <row r="75">
+      <c r="A75" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C75">
         <v>46132</v>
       </c>
@@ -6839,6 +6919,9 @@
       </c>
     </row>
     <row r="76">
+      <c r="A76" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C76">
         <v>46133</v>
       </c>
@@ -6856,6 +6939,9 @@
       </c>
     </row>
     <row r="77">
+      <c r="A77" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C77">
         <v>46134</v>
       </c>
@@ -6873,6 +6959,9 @@
       </c>
     </row>
     <row r="78">
+      <c r="A78" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C78">
         <v>46135</v>
       </c>
@@ -6890,6 +6979,9 @@
       </c>
     </row>
     <row r="79">
+      <c r="A79" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C79">
         <v>46135</v>
       </c>
@@ -6907,6 +6999,9 @@
       </c>
     </row>
     <row r="80">
+      <c r="A80" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C80">
         <v>46135</v>
       </c>
@@ -6924,6 +7019,9 @@
       </c>
     </row>
     <row r="81">
+      <c r="A81" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C81">
         <v>46136</v>
       </c>
@@ -6941,6 +7039,9 @@
       </c>
     </row>
     <row r="82">
+      <c r="A82" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C82">
         <v>46137</v>
       </c>
@@ -6958,6 +7059,9 @@
       </c>
     </row>
     <row r="83">
+      <c r="A83" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C83">
         <v>46138</v>
       </c>
@@ -6975,6 +7079,9 @@
       </c>
     </row>
     <row r="84">
+      <c r="A84" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C84">
         <v>46139</v>
       </c>
@@ -6992,6 +7099,9 @@
       </c>
     </row>
     <row r="85">
+      <c r="A85" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C85">
         <v>46140</v>
       </c>
@@ -7009,6 +7119,9 @@
       </c>
     </row>
     <row r="86">
+      <c r="A86" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C86">
         <v>46140</v>
       </c>
@@ -7026,6 +7139,9 @@
       </c>
     </row>
     <row r="87">
+      <c r="A87" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C87">
         <v>46141</v>
       </c>
@@ -7043,6 +7159,9 @@
       </c>
     </row>
     <row r="88">
+      <c r="A88" t="str">
+        <v>Abril</v>
+      </c>
       <c r="C88">
         <v>46142</v>
       </c>
@@ -7466,6 +7585,9 @@
       </c>
     </row>
     <row r="115">
+      <c r="A115" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C115">
         <v>46235</v>
       </c>
@@ -7483,6 +7605,9 @@
       </c>
     </row>
     <row r="116">
+      <c r="A116" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C116">
         <v>46236</v>
       </c>
@@ -7500,6 +7625,9 @@
       </c>
     </row>
     <row r="117">
+      <c r="A117" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C117">
         <v>46236</v>
       </c>
@@ -7517,6 +7645,9 @@
       </c>
     </row>
     <row r="118">
+      <c r="A118" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C118">
         <v>46237</v>
       </c>
@@ -7534,6 +7665,9 @@
       </c>
     </row>
     <row r="119">
+      <c r="A119" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C119">
         <v>46237</v>
       </c>
@@ -7551,6 +7685,9 @@
       </c>
     </row>
     <row r="120">
+      <c r="A120" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C120">
         <v>46238</v>
       </c>
@@ -7568,6 +7705,9 @@
       </c>
     </row>
     <row r="121">
+      <c r="A121" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C121">
         <v>46239</v>
       </c>
@@ -7585,6 +7725,9 @@
       </c>
     </row>
     <row r="122">
+      <c r="A122" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C122">
         <v>46240</v>
       </c>
@@ -7602,6 +7745,9 @@
       </c>
     </row>
     <row r="123">
+      <c r="A123" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C123">
         <v>46240</v>
       </c>
@@ -7619,6 +7765,9 @@
       </c>
     </row>
     <row r="124">
+      <c r="A124" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C124">
         <v>46240</v>
       </c>
@@ -7636,6 +7785,9 @@
       </c>
     </row>
     <row r="125">
+      <c r="A125" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C125">
         <v>46240</v>
       </c>
@@ -7653,6 +7805,9 @@
       </c>
     </row>
     <row r="126">
+      <c r="A126" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C126">
         <v>46241</v>
       </c>
@@ -7670,6 +7825,9 @@
       </c>
     </row>
     <row r="127">
+      <c r="A127" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C127">
         <v>46242</v>
       </c>
@@ -7687,6 +7845,9 @@
       </c>
     </row>
     <row r="128">
+      <c r="A128" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C128">
         <v>46244</v>
       </c>
@@ -7704,6 +7865,9 @@
       </c>
     </row>
     <row r="129">
+      <c r="A129" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C129">
         <v>46244</v>
       </c>
@@ -7721,6 +7885,9 @@
       </c>
     </row>
     <row r="130">
+      <c r="A130" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C130">
         <v>46244</v>
       </c>
@@ -7738,6 +7905,9 @@
       </c>
     </row>
     <row r="131">
+      <c r="A131" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C131">
         <v>46245</v>
       </c>
@@ -7755,6 +7925,9 @@
       </c>
     </row>
     <row r="132">
+      <c r="A132" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C132">
         <v>46245</v>
       </c>
@@ -7772,6 +7945,9 @@
       </c>
     </row>
     <row r="133">
+      <c r="A133" t="str">
+        <v>Agosto</v>
+      </c>
       <c r="C133">
         <v>46245</v>
       </c>

</xml_diff>

<commit_message>
Custos fixos futuros provisionados com status Pendente e vencimentos corretos
</commit_message>
<xml_diff>
--- a/Controle_Financeiro_2026.xlsx
+++ b/Controle_Financeiro_2026.xlsx
@@ -3209,7 +3209,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I136"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5490,67 +5490,899 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D98">
-        <v>2638.54</v>
+        <v>Setembro</v>
+      </c>
+      <c r="B98">
+        <v>46275</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F98" t="str">
+        <v>Estrutura</v>
+      </c>
+      <c r="G98">
+        <v>1000</v>
+      </c>
+      <c r="H98" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I98" t="str">
+        <v>Locação Estúdio / Espaço PJ</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D99">
-        <v>2111.89</v>
+        <v>Setembro</v>
+      </c>
+      <c r="B99">
+        <v>46267</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Google On</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F99" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G99">
+        <v>96.99</v>
+      </c>
+      <c r="H99" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I99" t="str">
+        <v>Armazenamento Nuvem</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D100">
-        <v>1751.89</v>
+        <v>Setembro</v>
+      </c>
+      <c r="B100">
+        <v>46275</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Adobe Creative Cloud</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F100" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G100">
+        <v>129</v>
+      </c>
+      <c r="H100" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I100" t="str">
+        <v>Plano Aplicativos Adobe</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D101">
-        <v>1751.89</v>
+        <v>Setembro</v>
+      </c>
+      <c r="B101">
+        <v>46275</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Contador / Honorários - Isabel Almeida</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F101" t="str">
+        <v>Contabilidade</v>
+      </c>
+      <c r="G101">
+        <v>400</v>
+      </c>
+      <c r="H101" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I101" t="str">
+        <v>Honorários Contábeis PJ</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D102">
-        <v>3601.89</v>
+        <v>Setembro</v>
+      </c>
+      <c r="B102">
+        <v>46285</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Canva Pro</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F102" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G102">
+        <v>47</v>
+      </c>
+      <c r="H102" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I102" t="str">
+        <v>Assinatura Canva</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>📊  TOTAIS POR CATEGORIA</v>
+        <v>Setembro</v>
+      </c>
+      <c r="B103">
+        <v>46280</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Amazon Prime / Digital</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F103" t="str">
+        <v>Serviços Digitais</v>
+      </c>
+      <c r="G103">
+        <v>54.8</v>
+      </c>
+      <c r="H103" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I103" t="str">
+        <v>Assinatura Serviços</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B104">
+        <v>46285</v>
+      </c>
+      <c r="D104" t="str">
+        <v>DAS Simples Nacional</v>
+      </c>
+      <c r="E104" t="str">
+        <v>Impostos e Taxas</v>
+      </c>
+      <c r="F104" t="str">
+        <v>Impostos</v>
+      </c>
+      <c r="G104">
+        <v>0</v>
+      </c>
+      <c r="H104" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I104" t="str">
+        <v>Aguardando apuração da contabilidade</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B105">
+        <v>46290</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Renegociação PJ</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F105" t="str">
+        <v>Dívidas PJ</v>
+      </c>
+      <c r="G105">
+        <v>60</v>
+      </c>
+      <c r="H105" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I105" t="str">
+        <v>Parcelamento PJ</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B106">
+        <v>46305</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F106" t="str">
+        <v>Estrutura</v>
+      </c>
+      <c r="G106">
+        <v>1000</v>
+      </c>
+      <c r="H106" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I106" t="str">
+        <v>Locação Estúdio / Espaço PJ</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B107">
+        <v>46297</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Google On</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F107" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G107">
+        <v>96.99</v>
+      </c>
+      <c r="H107" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I107" t="str">
+        <v>Armazenamento Nuvem</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B108">
+        <v>46305</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Adobe Creative Cloud</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F108" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G108">
+        <v>129</v>
+      </c>
+      <c r="H108" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I108" t="str">
+        <v>Plano Aplicativos Adobe</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B109">
+        <v>46305</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Contador / Honorários - Isabel Almeida</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F109" t="str">
+        <v>Contabilidade</v>
+      </c>
+      <c r="G109">
+        <v>400</v>
+      </c>
+      <c r="H109" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I109" t="str">
+        <v>Honorários Contábeis PJ</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B110">
+        <v>46315</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Canva Pro</v>
+      </c>
+      <c r="E110" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F110" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G110">
+        <v>47</v>
+      </c>
+      <c r="H110" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I110" t="str">
+        <v>Assinatura Canva</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B111">
+        <v>46310</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Amazon Prime / Digital</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F111" t="str">
+        <v>Serviços Digitais</v>
+      </c>
+      <c r="G111">
+        <v>54.8</v>
+      </c>
+      <c r="H111" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I111" t="str">
+        <v>Assinatura Serviços</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B112">
+        <v>46315</v>
+      </c>
+      <c r="D112" t="str">
+        <v>DAS Simples Nacional</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Impostos e Taxas</v>
+      </c>
+      <c r="F112" t="str">
+        <v>Impostos</v>
+      </c>
+      <c r="G112">
+        <v>0</v>
+      </c>
+      <c r="H112" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I112" t="str">
+        <v>Aguardando apuração da contabilidade</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B113">
+        <v>46320</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Renegociação PJ</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F113" t="str">
+        <v>Dívidas PJ</v>
+      </c>
+      <c r="G113">
+        <v>60</v>
+      </c>
+      <c r="H113" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I113" t="str">
+        <v>Parcelamento PJ</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B114">
+        <v>46336</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
+      </c>
+      <c r="E114" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F114" t="str">
+        <v>Estrutura</v>
+      </c>
+      <c r="G114">
+        <v>1000</v>
+      </c>
+      <c r="H114" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I114" t="str">
+        <v>Locação Estúdio / Espaço PJ</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B115">
+        <v>46328</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Google On</v>
+      </c>
+      <c r="E115" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F115" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G115">
+        <v>96.99</v>
+      </c>
+      <c r="H115" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I115" t="str">
+        <v>Armazenamento Nuvem</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B116">
+        <v>46336</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Adobe Creative Cloud</v>
+      </c>
+      <c r="E116" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F116" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G116">
+        <v>129</v>
+      </c>
+      <c r="H116" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I116" t="str">
+        <v>Plano Aplicativos Adobe</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B117">
+        <v>46336</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Contador / Honorários - Isabel Almeida</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F117" t="str">
+        <v>Contabilidade</v>
+      </c>
+      <c r="G117">
+        <v>400</v>
+      </c>
+      <c r="H117" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I117" t="str">
+        <v>Honorários Contábeis PJ</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B118">
+        <v>46346</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Canva Pro</v>
+      </c>
+      <c r="E118" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F118" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G118">
+        <v>47</v>
+      </c>
+      <c r="H118" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I118" t="str">
+        <v>Assinatura Canva</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B119">
+        <v>46341</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Amazon Prime / Digital</v>
+      </c>
+      <c r="E119" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F119" t="str">
+        <v>Serviços Digitais</v>
+      </c>
+      <c r="G119">
+        <v>54.8</v>
+      </c>
+      <c r="H119" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I119" t="str">
+        <v>Assinatura Serviços</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B120">
+        <v>46346</v>
+      </c>
+      <c r="D120" t="str">
+        <v>DAS Simples Nacional</v>
+      </c>
+      <c r="E120" t="str">
+        <v>Impostos e Taxas</v>
+      </c>
+      <c r="F120" t="str">
+        <v>Impostos</v>
+      </c>
+      <c r="G120">
+        <v>0</v>
+      </c>
+      <c r="H120" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I120" t="str">
+        <v>Aguardando apuração da contabilidade</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B121">
+        <v>46351</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Renegociação PJ</v>
+      </c>
+      <c r="E121" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F121" t="str">
+        <v>Dívidas PJ</v>
+      </c>
+      <c r="G121">
+        <v>60</v>
+      </c>
+      <c r="H121" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I121" t="str">
+        <v>Parcelamento PJ</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B122">
+        <v>46366</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Aluguel do Estúdio (Julio Cesar Paz)</v>
+      </c>
+      <c r="E122" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F122" t="str">
+        <v>Estrutura</v>
+      </c>
+      <c r="G122">
+        <v>1000</v>
+      </c>
+      <c r="H122" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I122" t="str">
+        <v>Locação Estúdio / Espaço PJ</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B123">
+        <v>46358</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Google On</v>
+      </c>
+      <c r="E123" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F123" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G123">
+        <v>96.99</v>
+      </c>
+      <c r="H123" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I123" t="str">
+        <v>Armazenamento Nuvem</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B124">
+        <v>46366</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Adobe Creative Cloud</v>
+      </c>
+      <c r="E124" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F124" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G124">
+        <v>129</v>
+      </c>
+      <c r="H124" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I124" t="str">
+        <v>Plano Aplicativos Adobe</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B125">
+        <v>46366</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Contador / Honorários - Isabel Almeida</v>
+      </c>
+      <c r="E125" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F125" t="str">
+        <v>Contabilidade</v>
+      </c>
+      <c r="G125">
+        <v>400</v>
+      </c>
+      <c r="H125" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I125" t="str">
+        <v>Honorários Contábeis PJ</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B126">
+        <v>46376</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Canva Pro</v>
+      </c>
+      <c r="E126" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F126" t="str">
+        <v>Softwares</v>
+      </c>
+      <c r="G126">
+        <v>47</v>
+      </c>
+      <c r="H126" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I126" t="str">
+        <v>Assinatura Canva</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B127">
+        <v>46371</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Amazon Prime / Digital</v>
+      </c>
+      <c r="E127" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F127" t="str">
+        <v>Serviços Digitais</v>
+      </c>
+      <c r="G127">
+        <v>54.8</v>
+      </c>
+      <c r="H127" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I127" t="str">
+        <v>Assinatura Serviços</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B128">
+        <v>46376</v>
+      </c>
+      <c r="D128" t="str">
+        <v>DAS Simples Nacional</v>
+      </c>
+      <c r="E128" t="str">
+        <v>Impostos e Taxas</v>
+      </c>
+      <c r="F128" t="str">
+        <v>Impostos</v>
+      </c>
+      <c r="G128">
+        <v>0</v>
+      </c>
+      <c r="H128" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I128" t="str">
+        <v>Aguardando apuração da contabilidade</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B129">
+        <v>46381</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Renegociação PJ</v>
+      </c>
+      <c r="E129" t="str">
+        <v>Custos Fixos</v>
+      </c>
+      <c r="F129" t="str">
+        <v>Dívidas PJ</v>
+      </c>
+      <c r="G129">
+        <v>60</v>
+      </c>
+      <c r="H129" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="I129" t="str">
+        <v>Parcelamento PJ</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>Total</v>
+      </c>
+      <c r="D130">
+        <v>2638.54</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>Total</v>
+      </c>
+      <c r="D131">
+        <v>2111.89</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>Total</v>
+      </c>
+      <c r="D132">
+        <v>1751.89</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>Total</v>
+      </c>
+      <c r="D133">
+        <v>1751.89</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>Total</v>
+      </c>
+      <c r="D134">
+        <v>3601.89</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>📊  TOTAIS POR CATEGORIA</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
         <v>💰 TOTAL GERAL EMPRESA</v>
       </c>
-      <c r="G104">
+      <c r="G136">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I104"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I136"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H277"/>
+  <dimension ref="A1:H337"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11503,31 +12335,1411 @@
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D275">
-        <v>0</v>
+        <v>Setembro</v>
+      </c>
+      <c r="B275">
+        <v>46275</v>
+      </c>
+      <c r="D275" t="str">
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+      </c>
+      <c r="E275" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F275">
+        <v>1300</v>
+      </c>
+      <c r="G275" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H275" t="str">
+        <v>Aluguel residencial parcela 1</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D276">
-        <v>415.18</v>
+        <v>Setembro</v>
+      </c>
+      <c r="B276">
+        <v>46290</v>
+      </c>
+      <c r="D276" t="str">
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+      </c>
+      <c r="E276" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F276">
+        <v>700</v>
+      </c>
+      <c r="G276" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H276" t="str">
+        <v>Aluguel residencial parcela 2</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B277">
+        <v>46275</v>
+      </c>
+      <c r="D277" t="str">
+        <v>IPTU (parcela mensal) Lusitania</v>
+      </c>
+      <c r="E277" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F277">
+        <v>290</v>
+      </c>
+      <c r="G277" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H277" t="str">
+        <v>Parcela IPTU residencial</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B278">
+        <v>46277</v>
+      </c>
+      <c r="D278" t="str">
+        <v>Diarista / Limpeza - Maria Auxiliadora (1/2)</v>
+      </c>
+      <c r="E278" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F278">
+        <v>440</v>
+      </c>
+      <c r="G278" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H278" t="str">
+        <v>Diárias limpeza quinzena 1</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B279">
+        <v>46291</v>
+      </c>
+      <c r="D279" t="str">
+        <v>Diarista / Limpeza - Maria Auxiliadora (2/2)</v>
+      </c>
+      <c r="E279" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F279">
+        <v>220</v>
+      </c>
+      <c r="G279" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H279" t="str">
+        <v>Diária limpeza quinzena 2</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B280">
+        <v>46291</v>
+      </c>
+      <c r="D280" t="str">
+        <v>Diarista / Limpeza - Rosana Francelino</v>
+      </c>
+      <c r="E280" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F280">
+        <v>220</v>
+      </c>
+      <c r="G280" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H280" t="str">
+        <v>Diária limpeza quinzena 2</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B281">
+        <v>46270</v>
+      </c>
+      <c r="D281" t="str">
+        <v>Vivo Telefonia &amp; Internet</v>
+      </c>
+      <c r="E281" t="str">
+        <v>Serviços</v>
+      </c>
+      <c r="F281">
+        <v>481.63</v>
+      </c>
+      <c r="G281" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H281" t="str">
+        <v>Linha celular e internet residencial</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B282">
+        <v>46280</v>
+      </c>
+      <c r="D282" t="str">
+        <v>Ajuda Familiar (Tia via Douglas)</v>
+      </c>
+      <c r="E282" t="str">
+        <v>Família</v>
+      </c>
+      <c r="F282">
+        <v>150</v>
+      </c>
+      <c r="G282" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H282" t="str">
+        <v>Dinheiro enviado para a Tia via Douglas</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B283">
+        <v>46285</v>
+      </c>
+      <c r="D283" t="str">
+        <v>Ajuda Familiar (Tia via Douglas)</v>
+      </c>
+      <c r="E283" t="str">
+        <v>Família</v>
+      </c>
+      <c r="F283">
+        <v>200</v>
+      </c>
+      <c r="G283" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H283" t="str">
+        <v>Dinheiro enviado para a Tia via Douglas</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B284">
+        <v>46275</v>
+      </c>
+      <c r="D284" t="str">
+        <v>Nu Seguro Celular</v>
+      </c>
+      <c r="E284" t="str">
+        <v>Serviços</v>
+      </c>
+      <c r="F284">
+        <v>66.12</v>
+      </c>
+      <c r="G284" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H284" t="str">
+        <v>Seguro celular</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B285">
+        <v>46289</v>
+      </c>
+      <c r="D285" t="str">
+        <v>Sócio Torcedor Flamengo</v>
+      </c>
+      <c r="E285" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F285">
+        <v>312</v>
+      </c>
+      <c r="G285" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H285" t="str">
+        <v>Sócio torcedor CRF</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B286">
+        <v>46289</v>
+      </c>
+      <c r="D286" t="str">
+        <v>Netflix</v>
+      </c>
+      <c r="E286" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F286">
+        <v>20.9</v>
+      </c>
+      <c r="G286" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H286" t="str">
+        <v>Assinatura Netflix</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B287">
+        <v>46285</v>
+      </c>
+      <c r="D287" t="str">
+        <v>YouTube Premium</v>
+      </c>
+      <c r="E287" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F287">
+        <v>25.92</v>
+      </c>
+      <c r="G287" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H287" t="str">
+        <v>Assinatura YouTube</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B288">
+        <v>46267</v>
+      </c>
+      <c r="D288" t="str">
+        <v>Clube iFood</v>
+      </c>
+      <c r="E288" t="str">
+        <v>Alimentação</v>
+      </c>
+      <c r="F288">
+        <v>5.95</v>
+      </c>
+      <c r="G288" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H288" t="str">
+        <v>Assinatura Clube iFood</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>Setembro</v>
+      </c>
+      <c r="B289">
+        <v>46275</v>
+      </c>
+      <c r="D289" t="str">
+        <v>Condomínio Citta America</v>
+      </c>
+      <c r="E289" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F289">
+        <v>51.6</v>
+      </c>
+      <c r="G289" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H289" t="str">
+        <v>Taxa condomínio / garagem</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B290">
+        <v>46305</v>
+      </c>
+      <c r="D290" t="str">
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+      </c>
+      <c r="E290" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F290">
+        <v>1300</v>
+      </c>
+      <c r="G290" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H290" t="str">
+        <v>Aluguel residencial parcela 1</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B291">
+        <v>46320</v>
+      </c>
+      <c r="D291" t="str">
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+      </c>
+      <c r="E291" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F291">
+        <v>700</v>
+      </c>
+      <c r="G291" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H291" t="str">
+        <v>Aluguel residencial parcela 2</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B292">
+        <v>46305</v>
+      </c>
+      <c r="D292" t="str">
+        <v>IPTU (parcela mensal) Lusitania</v>
+      </c>
+      <c r="E292" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F292">
+        <v>290</v>
+      </c>
+      <c r="G292" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H292" t="str">
+        <v>Parcela IPTU residencial</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B293">
+        <v>46307</v>
+      </c>
+      <c r="D293" t="str">
+        <v>Diarista / Limpeza - Maria Auxiliadora (1/2)</v>
+      </c>
+      <c r="E293" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F293">
+        <v>440</v>
+      </c>
+      <c r="G293" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H293" t="str">
+        <v>Diárias limpeza quinzena 1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B294">
+        <v>46321</v>
+      </c>
+      <c r="D294" t="str">
+        <v>Diarista / Limpeza - Maria Auxiliadora (2/2)</v>
+      </c>
+      <c r="E294" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F294">
+        <v>220</v>
+      </c>
+      <c r="G294" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H294" t="str">
+        <v>Diária limpeza quinzena 2</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B295">
+        <v>46321</v>
+      </c>
+      <c r="D295" t="str">
+        <v>Diarista / Limpeza - Rosana Francelino</v>
+      </c>
+      <c r="E295" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F295">
+        <v>220</v>
+      </c>
+      <c r="G295" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H295" t="str">
+        <v>Diária limpeza quinzena 2</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B296">
+        <v>46300</v>
+      </c>
+      <c r="D296" t="str">
+        <v>Vivo Telefonia &amp; Internet</v>
+      </c>
+      <c r="E296" t="str">
+        <v>Serviços</v>
+      </c>
+      <c r="F296">
+        <v>481.63</v>
+      </c>
+      <c r="G296" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H296" t="str">
+        <v>Linha celular e internet residencial</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B297">
+        <v>46310</v>
+      </c>
+      <c r="D297" t="str">
+        <v>Ajuda Familiar (Tia via Douglas)</v>
+      </c>
+      <c r="E297" t="str">
+        <v>Família</v>
+      </c>
+      <c r="F297">
+        <v>150</v>
+      </c>
+      <c r="G297" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H297" t="str">
+        <v>Dinheiro enviado para a Tia via Douglas</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B298">
+        <v>46315</v>
+      </c>
+      <c r="D298" t="str">
+        <v>Ajuda Familiar (Tia via Douglas)</v>
+      </c>
+      <c r="E298" t="str">
+        <v>Família</v>
+      </c>
+      <c r="F298">
+        <v>200</v>
+      </c>
+      <c r="G298" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H298" t="str">
+        <v>Dinheiro enviado para a Tia via Douglas</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B299">
+        <v>46305</v>
+      </c>
+      <c r="D299" t="str">
+        <v>Nu Seguro Celular</v>
+      </c>
+      <c r="E299" t="str">
+        <v>Serviços</v>
+      </c>
+      <c r="F299">
+        <v>66.12</v>
+      </c>
+      <c r="G299" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H299" t="str">
+        <v>Seguro celular</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B300">
+        <v>46319</v>
+      </c>
+      <c r="D300" t="str">
+        <v>Sócio Torcedor Flamengo</v>
+      </c>
+      <c r="E300" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F300">
+        <v>312</v>
+      </c>
+      <c r="G300" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H300" t="str">
+        <v>Sócio torcedor CRF</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B301">
+        <v>46319</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Netflix</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F301">
+        <v>20.9</v>
+      </c>
+      <c r="G301" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H301" t="str">
+        <v>Assinatura Netflix</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B302">
+        <v>46315</v>
+      </c>
+      <c r="D302" t="str">
+        <v>YouTube Premium</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F302">
+        <v>25.92</v>
+      </c>
+      <c r="G302" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H302" t="str">
+        <v>Assinatura YouTube</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B303">
+        <v>46297</v>
+      </c>
+      <c r="D303" t="str">
+        <v>Clube iFood</v>
+      </c>
+      <c r="E303" t="str">
+        <v>Alimentação</v>
+      </c>
+      <c r="F303">
+        <v>5.95</v>
+      </c>
+      <c r="G303" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H303" t="str">
+        <v>Assinatura Clube iFood</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>Outubro</v>
+      </c>
+      <c r="B304">
+        <v>46305</v>
+      </c>
+      <c r="D304" t="str">
+        <v>Condomínio Citta America</v>
+      </c>
+      <c r="E304" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F304">
+        <v>51.6</v>
+      </c>
+      <c r="G304" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H304" t="str">
+        <v>Taxa condomínio / garagem</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B305">
+        <v>46336</v>
+      </c>
+      <c r="D305" t="str">
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+      </c>
+      <c r="E305" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F305">
+        <v>1300</v>
+      </c>
+      <c r="G305" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H305" t="str">
+        <v>Aluguel residencial parcela 1</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B306">
+        <v>46351</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F306">
+        <v>700</v>
+      </c>
+      <c r="G306" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H306" t="str">
+        <v>Aluguel residencial parcela 2</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B307">
+        <v>46336</v>
+      </c>
+      <c r="D307" t="str">
+        <v>IPTU (parcela mensal) Lusitania</v>
+      </c>
+      <c r="E307" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F307">
+        <v>290</v>
+      </c>
+      <c r="G307" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H307" t="str">
+        <v>Parcela IPTU residencial</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B308">
+        <v>46338</v>
+      </c>
+      <c r="D308" t="str">
+        <v>Diarista / Limpeza - Maria Auxiliadora (1/2)</v>
+      </c>
+      <c r="E308" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F308">
+        <v>440</v>
+      </c>
+      <c r="G308" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H308" t="str">
+        <v>Diárias limpeza quinzena 1</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B309">
+        <v>46352</v>
+      </c>
+      <c r="D309" t="str">
+        <v>Diarista / Limpeza - Maria Auxiliadora (2/2)</v>
+      </c>
+      <c r="E309" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F309">
+        <v>220</v>
+      </c>
+      <c r="G309" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H309" t="str">
+        <v>Diária limpeza quinzena 2</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B310">
+        <v>46352</v>
+      </c>
+      <c r="D310" t="str">
+        <v>Diarista / Limpeza - Rosana Francelino</v>
+      </c>
+      <c r="E310" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F310">
+        <v>220</v>
+      </c>
+      <c r="G310" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H310" t="str">
+        <v>Diária limpeza quinzena 2</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B311">
+        <v>46331</v>
+      </c>
+      <c r="D311" t="str">
+        <v>Vivo Telefonia &amp; Internet</v>
+      </c>
+      <c r="E311" t="str">
+        <v>Serviços</v>
+      </c>
+      <c r="F311">
+        <v>481.63</v>
+      </c>
+      <c r="G311" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H311" t="str">
+        <v>Linha celular e internet residencial</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B312">
+        <v>46341</v>
+      </c>
+      <c r="D312" t="str">
+        <v>Ajuda Familiar (Tia via Douglas)</v>
+      </c>
+      <c r="E312" t="str">
+        <v>Família</v>
+      </c>
+      <c r="F312">
+        <v>150</v>
+      </c>
+      <c r="G312" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H312" t="str">
+        <v>Dinheiro enviado para a Tia via Douglas</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B313">
+        <v>46346</v>
+      </c>
+      <c r="D313" t="str">
+        <v>Ajuda Familiar (Tia via Douglas)</v>
+      </c>
+      <c r="E313" t="str">
+        <v>Família</v>
+      </c>
+      <c r="F313">
+        <v>200</v>
+      </c>
+      <c r="G313" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H313" t="str">
+        <v>Dinheiro enviado para a Tia via Douglas</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B314">
+        <v>46336</v>
+      </c>
+      <c r="D314" t="str">
+        <v>Nu Seguro Celular</v>
+      </c>
+      <c r="E314" t="str">
+        <v>Serviços</v>
+      </c>
+      <c r="F314">
+        <v>66.12</v>
+      </c>
+      <c r="G314" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H314" t="str">
+        <v>Seguro celular</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B315">
+        <v>46350</v>
+      </c>
+      <c r="D315" t="str">
+        <v>Sócio Torcedor Flamengo</v>
+      </c>
+      <c r="E315" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F315">
+        <v>312</v>
+      </c>
+      <c r="G315" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H315" t="str">
+        <v>Sócio torcedor CRF</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B316">
+        <v>46350</v>
+      </c>
+      <c r="D316" t="str">
+        <v>Netflix</v>
+      </c>
+      <c r="E316" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F316">
+        <v>20.9</v>
+      </c>
+      <c r="G316" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H316" t="str">
+        <v>Assinatura Netflix</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B317">
+        <v>46346</v>
+      </c>
+      <c r="D317" t="str">
+        <v>YouTube Premium</v>
+      </c>
+      <c r="E317" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F317">
+        <v>25.92</v>
+      </c>
+      <c r="G317" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H317" t="str">
+        <v>Assinatura YouTube</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B318">
+        <v>46328</v>
+      </c>
+      <c r="D318" t="str">
+        <v>Clube iFood</v>
+      </c>
+      <c r="E318" t="str">
+        <v>Alimentação</v>
+      </c>
+      <c r="F318">
+        <v>5.95</v>
+      </c>
+      <c r="G318" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H318" t="str">
+        <v>Assinatura Clube iFood</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>Novembro</v>
+      </c>
+      <c r="B319">
+        <v>46336</v>
+      </c>
+      <c r="D319" t="str">
+        <v>Condomínio Citta America</v>
+      </c>
+      <c r="E319" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F319">
+        <v>51.6</v>
+      </c>
+      <c r="G319" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H319" t="str">
+        <v>Taxa condomínio / garagem</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B320">
+        <v>46366</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+      </c>
+      <c r="E320" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F320">
+        <v>1300</v>
+      </c>
+      <c r="G320" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H320" t="str">
+        <v>Aluguel residencial parcela 1</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B321">
+        <v>46381</v>
+      </c>
+      <c r="D321" t="str">
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+      </c>
+      <c r="E321" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F321">
+        <v>700</v>
+      </c>
+      <c r="G321" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H321" t="str">
+        <v>Aluguel residencial parcela 2</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B322">
+        <v>46366</v>
+      </c>
+      <c r="D322" t="str">
+        <v>IPTU (parcela mensal) Lusitania</v>
+      </c>
+      <c r="E322" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F322">
+        <v>290</v>
+      </c>
+      <c r="G322" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H322" t="str">
+        <v>Parcela IPTU residencial</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B323">
+        <v>46368</v>
+      </c>
+      <c r="D323" t="str">
+        <v>Diarista / Limpeza - Maria Auxiliadora (1/2)</v>
+      </c>
+      <c r="E323" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F323">
+        <v>440</v>
+      </c>
+      <c r="G323" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H323" t="str">
+        <v>Diárias limpeza quinzena 1</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B324">
+        <v>46382</v>
+      </c>
+      <c r="D324" t="str">
+        <v>Diarista / Limpeza - Maria Auxiliadora (2/2)</v>
+      </c>
+      <c r="E324" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F324">
+        <v>220</v>
+      </c>
+      <c r="G324" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H324" t="str">
+        <v>Diária limpeza quinzena 2</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B325">
+        <v>46382</v>
+      </c>
+      <c r="D325" t="str">
+        <v>Diarista / Limpeza - Rosana Francelino</v>
+      </c>
+      <c r="E325" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F325">
+        <v>220</v>
+      </c>
+      <c r="G325" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H325" t="str">
+        <v>Diária limpeza quinzena 2</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B326">
+        <v>46361</v>
+      </c>
+      <c r="D326" t="str">
+        <v>Vivo Telefonia &amp; Internet</v>
+      </c>
+      <c r="E326" t="str">
+        <v>Serviços</v>
+      </c>
+      <c r="F326">
+        <v>481.63</v>
+      </c>
+      <c r="G326" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H326" t="str">
+        <v>Linha celular e internet residencial</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B327">
+        <v>46371</v>
+      </c>
+      <c r="D327" t="str">
+        <v>Ajuda Familiar (Tia via Douglas)</v>
+      </c>
+      <c r="E327" t="str">
+        <v>Família</v>
+      </c>
+      <c r="F327">
+        <v>150</v>
+      </c>
+      <c r="G327" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H327" t="str">
+        <v>Dinheiro enviado para a Tia via Douglas</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B328">
+        <v>46376</v>
+      </c>
+      <c r="D328" t="str">
+        <v>Ajuda Familiar (Tia via Douglas)</v>
+      </c>
+      <c r="E328" t="str">
+        <v>Família</v>
+      </c>
+      <c r="F328">
+        <v>200</v>
+      </c>
+      <c r="G328" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H328" t="str">
+        <v>Dinheiro enviado para a Tia via Douglas</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B329">
+        <v>46366</v>
+      </c>
+      <c r="D329" t="str">
+        <v>Nu Seguro Celular</v>
+      </c>
+      <c r="E329" t="str">
+        <v>Serviços</v>
+      </c>
+      <c r="F329">
+        <v>66.12</v>
+      </c>
+      <c r="G329" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H329" t="str">
+        <v>Seguro celular</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B330">
+        <v>46380</v>
+      </c>
+      <c r="D330" t="str">
+        <v>Sócio Torcedor Flamengo</v>
+      </c>
+      <c r="E330" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F330">
+        <v>312</v>
+      </c>
+      <c r="G330" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H330" t="str">
+        <v>Sócio torcedor CRF</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B331">
+        <v>46380</v>
+      </c>
+      <c r="D331" t="str">
+        <v>Netflix</v>
+      </c>
+      <c r="E331" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F331">
+        <v>20.9</v>
+      </c>
+      <c r="G331" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H331" t="str">
+        <v>Assinatura Netflix</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B332">
+        <v>46376</v>
+      </c>
+      <c r="D332" t="str">
+        <v>YouTube Premium</v>
+      </c>
+      <c r="E332" t="str">
+        <v>Lazer &amp; Assinaturas</v>
+      </c>
+      <c r="F332">
+        <v>25.92</v>
+      </c>
+      <c r="G332" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H332" t="str">
+        <v>Assinatura YouTube</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B333">
+        <v>46358</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Clube iFood</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Alimentação</v>
+      </c>
+      <c r="F333">
+        <v>5.95</v>
+      </c>
+      <c r="G333" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H333" t="str">
+        <v>Assinatura Clube iFood</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>Dezembro</v>
+      </c>
+      <c r="B334">
+        <v>46366</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Condomínio Citta America</v>
+      </c>
+      <c r="E334" t="str">
+        <v>Moradia</v>
+      </c>
+      <c r="F334">
+        <v>51.6</v>
+      </c>
+      <c r="G334" t="str">
+        <v>⏳ Pendente</v>
+      </c>
+      <c r="H334" t="str">
+        <v>Taxa condomínio / garagem</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>Total</v>
+      </c>
+      <c r="D335">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>Total</v>
+      </c>
+      <c r="D336">
+        <v>415.18</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
         <v>💰 TOTAL GERAL PESSOAL</v>
       </c>
-      <c r="F277">
+      <c r="F337">
         <v>2622.22</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H277"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H337"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Zerar valor de Renegociação PJ em todos os meses
</commit_message>
<xml_diff>
--- a/Controle_Financeiro_2026.xlsx
+++ b/Controle_Financeiro_2026.xlsx
@@ -3441,7 +3441,7 @@
         <v>Custos Fixos</v>
       </c>
       <c r="G14">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3773,7 +3773,7 @@
         <v>Custos Fixos</v>
       </c>
       <c r="G33">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -4319,7 +4319,7 @@
         <v>Dívidas PJ</v>
       </c>
       <c r="G57">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H57" t="str">
         <v>⏳ Pendente</v>
@@ -5687,7 +5687,7 @@
         <v>Dívidas PJ</v>
       </c>
       <c r="G105">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H105" t="str">
         <v>⏳ Pendente</v>
@@ -5895,7 +5895,7 @@
         <v>Dívidas PJ</v>
       </c>
       <c r="G113">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H113" t="str">
         <v>⏳ Pendente</v>
@@ -6103,7 +6103,7 @@
         <v>Dívidas PJ</v>
       </c>
       <c r="G121">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H121" t="str">
         <v>⏳ Pendente</v>
@@ -6311,7 +6311,7 @@
         <v>Dívidas PJ</v>
       </c>
       <c r="G129">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H129" t="str">
         <v>⏳ Pendente</v>

</xml_diff>

<commit_message>
Dashboard e aba Pessoal atualizados com projecoes de despesas fixas para todos os meses
</commit_message>
<xml_diff>
--- a/Controle_Financeiro_2026.xlsx
+++ b/Controle_Financeiro_2026.xlsx
@@ -426,6 +426,18 @@
       <c r="A2" t="str">
         <v>Empresa + Finanças Pessoais · Prestação de Serviços</v>
       </c>
+      <c r="J2">
+        <v>547.75</v>
+      </c>
+      <c r="K2">
+        <v>547.75</v>
+      </c>
+      <c r="L2">
+        <v>547.75</v>
+      </c>
+      <c r="M2">
+        <v>547.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -505,16 +517,16 @@
         <v>1577.79</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>1727.79</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>1727.79</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>1727.79</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>1727.79</v>
       </c>
       <c r="N6">
         <v>4057.81</v>
@@ -681,16 +693,16 @@
         <v>4254.67</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>1727.79</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>1727.79</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>1727.79</v>
       </c>
       <c r="M10">
-        <v>0</v>
+        <v>1727.79</v>
       </c>
       <c r="N10">
         <v>4220.7</v>
@@ -774,16 +786,16 @@
         <v>0</v>
       </c>
       <c r="J14">
-        <v>0</v>
+        <v>3221.6</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>3221.6</v>
       </c>
       <c r="L14">
-        <v>0</v>
+        <v>3221.6</v>
       </c>
       <c r="M14">
-        <v>0</v>
+        <v>3221.6</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -818,16 +830,16 @@
         <v>0</v>
       </c>
       <c r="J15">
-        <v>0</v>
+        <v>5.95</v>
       </c>
       <c r="K15">
-        <v>0</v>
+        <v>5.95</v>
       </c>
       <c r="L15">
-        <v>0</v>
+        <v>5.95</v>
       </c>
       <c r="M15">
-        <v>0</v>
+        <v>5.95</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -862,16 +874,16 @@
         <v>0</v>
       </c>
       <c r="J16">
-        <v>0</v>
+        <v>547.75</v>
       </c>
       <c r="K16">
-        <v>0</v>
+        <v>547.75</v>
       </c>
       <c r="L16">
-        <v>0</v>
+        <v>547.75</v>
       </c>
       <c r="M16">
-        <v>0</v>
+        <v>547.75</v>
       </c>
       <c r="N16">
         <v>0</v>
@@ -1038,16 +1050,16 @@
         <v>0</v>
       </c>
       <c r="J20">
-        <v>0</v>
+        <v>364.77</v>
       </c>
       <c r="K20">
-        <v>0</v>
+        <v>364.77</v>
       </c>
       <c r="L20">
-        <v>0</v>
+        <v>364.77</v>
       </c>
       <c r="M20">
-        <v>0</v>
+        <v>364.77</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -1170,16 +1182,16 @@
         <v>7613.08</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>4484.12</v>
       </c>
       <c r="K23">
-        <v>0</v>
+        <v>4484.12</v>
       </c>
       <c r="L23">
-        <v>0</v>
+        <v>4484.12</v>
       </c>
       <c r="M23">
-        <v>0</v>
+        <v>4484.12</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -1219,16 +1231,16 @@
         <v>11867.75</v>
       </c>
       <c r="J26">
-        <v>0</v>
+        <v>6211.91</v>
       </c>
       <c r="K26">
-        <v>0</v>
+        <v>6211.91</v>
       </c>
       <c r="L26">
-        <v>0</v>
+        <v>6211.91</v>
       </c>
       <c r="M26">
-        <v>0</v>
+        <v>6211.91</v>
       </c>
       <c r="N26">
         <v>4220.7</v>
@@ -1429,16 +1441,16 @@
         <v>1472.09</v>
       </c>
       <c r="J39">
-        <v>0</v>
+        <v>1472.09</v>
       </c>
       <c r="K39">
-        <v>0</v>
+        <v>1472.09</v>
       </c>
       <c r="L39">
-        <v>0</v>
+        <v>1472.09</v>
       </c>
       <c r="M39">
-        <v>0</v>
+        <v>1472.09</v>
       </c>
       <c r="N39">
         <v>4366.46</v>

</xml_diff>

<commit_message>
Ajuste diaristas 2x por semana (R$ 1.760/mes) e remocao de despesas eventuais dos fixos
</commit_message>
<xml_diff>
--- a/Controle_Financeiro_2026.xlsx
+++ b/Controle_Financeiro_2026.xlsx
@@ -786,16 +786,16 @@
         <v>0</v>
       </c>
       <c r="J14">
-        <v>3221.6</v>
+        <v>4050</v>
       </c>
       <c r="K14">
-        <v>3221.6</v>
+        <v>4050</v>
       </c>
       <c r="L14">
-        <v>3221.6</v>
+        <v>4050</v>
       </c>
       <c r="M14">
-        <v>3221.6</v>
+        <v>4050</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -1050,16 +1050,16 @@
         <v>0</v>
       </c>
       <c r="J20">
-        <v>364.77</v>
+        <v>46.82</v>
       </c>
       <c r="K20">
-        <v>364.77</v>
+        <v>46.82</v>
       </c>
       <c r="L20">
-        <v>364.77</v>
+        <v>46.82</v>
       </c>
       <c r="M20">
-        <v>364.77</v>
+        <v>46.82</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -1182,16 +1182,16 @@
         <v>7613.08</v>
       </c>
       <c r="J23">
-        <v>4484.12</v>
+        <v>4997.52</v>
       </c>
       <c r="K23">
-        <v>4484.12</v>
+        <v>4997.52</v>
       </c>
       <c r="L23">
-        <v>4484.12</v>
+        <v>4997.52</v>
       </c>
       <c r="M23">
-        <v>4484.12</v>
+        <v>4997.52</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -1231,16 +1231,16 @@
         <v>11867.75</v>
       </c>
       <c r="J26">
-        <v>6211.91</v>
+        <v>6725.31</v>
       </c>
       <c r="K26">
-        <v>6211.91</v>
+        <v>6725.31</v>
       </c>
       <c r="L26">
-        <v>6211.91</v>
+        <v>6725.31</v>
       </c>
       <c r="M26">
-        <v>6211.91</v>
+        <v>6725.31</v>
       </c>
       <c r="N26">
         <v>4220.7</v>
@@ -6394,7 +6394,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H337"/>
+  <dimension ref="A1:H333"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12419,10 +12419,10 @@
         <v>Setembro</v>
       </c>
       <c r="B278">
-        <v>46277</v>
+        <v>46270</v>
       </c>
       <c r="D278" t="str">
-        <v>Diarista / Limpeza - Maria Auxiliadora (1/2)</v>
+        <v>Diarista / Limpeza - Semana 1 (2 diárias)</v>
       </c>
       <c r="E278" t="str">
         <v>Moradia</v>
@@ -12434,7 +12434,7 @@
         <v>⏳ Pendente</v>
       </c>
       <c r="H278" t="str">
-        <v>Diárias limpeza quinzena 1</v>
+        <v>2 diárias de R$ 220 (Semana 1)</v>
       </c>
     </row>
     <row r="279">
@@ -12442,22 +12442,22 @@
         <v>Setembro</v>
       </c>
       <c r="B279">
-        <v>46291</v>
+        <v>46277</v>
       </c>
       <c r="D279" t="str">
-        <v>Diarista / Limpeza - Maria Auxiliadora (2/2)</v>
+        <v>Diarista / Limpeza - Semana 2 (2 diárias)</v>
       </c>
       <c r="E279" t="str">
         <v>Moradia</v>
       </c>
       <c r="F279">
-        <v>220</v>
+        <v>440</v>
       </c>
       <c r="G279" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H279" t="str">
-        <v>Diária limpeza quinzena 2</v>
+        <v>2 diárias de R$ 220 (Semana 2)</v>
       </c>
     </row>
     <row r="280">
@@ -12465,22 +12465,22 @@
         <v>Setembro</v>
       </c>
       <c r="B280">
-        <v>46291</v>
+        <v>46284</v>
       </c>
       <c r="D280" t="str">
-        <v>Diarista / Limpeza - Rosana Francelino</v>
+        <v>Diarista / Limpeza - Semana 3 (2 diárias)</v>
       </c>
       <c r="E280" t="str">
         <v>Moradia</v>
       </c>
       <c r="F280">
-        <v>220</v>
+        <v>440</v>
       </c>
       <c r="G280" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H280" t="str">
-        <v>Diária limpeza quinzena 2</v>
+        <v>2 diárias de R$ 220 (Semana 3)</v>
       </c>
     </row>
     <row r="281">
@@ -12488,22 +12488,22 @@
         <v>Setembro</v>
       </c>
       <c r="B281">
-        <v>46270</v>
+        <v>46291</v>
       </c>
       <c r="D281" t="str">
-        <v>Vivo Telefonia &amp; Internet</v>
+        <v>Diarista / Limpeza - Semana 4 (2 diárias)</v>
       </c>
       <c r="E281" t="str">
-        <v>Serviços</v>
+        <v>Moradia</v>
       </c>
       <c r="F281">
-        <v>481.63</v>
+        <v>440</v>
       </c>
       <c r="G281" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H281" t="str">
-        <v>Linha celular e internet residencial</v>
+        <v>2 diárias de R$ 220 (Semana 4)</v>
       </c>
     </row>
     <row r="282">
@@ -12511,22 +12511,22 @@
         <v>Setembro</v>
       </c>
       <c r="B282">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="D282" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>Vivo Telefonia &amp; Internet</v>
       </c>
       <c r="E282" t="str">
-        <v>Família</v>
+        <v>Serviços</v>
       </c>
       <c r="F282">
-        <v>150</v>
+        <v>481.63</v>
       </c>
       <c r="G282" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H282" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Linha celular e internet residencial</v>
       </c>
     </row>
     <row r="283">
@@ -12534,22 +12534,22 @@
         <v>Setembro</v>
       </c>
       <c r="B283">
-        <v>46285</v>
+        <v>46275</v>
       </c>
       <c r="D283" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>Nu Seguro Celular</v>
       </c>
       <c r="E283" t="str">
-        <v>Família</v>
+        <v>Serviços</v>
       </c>
       <c r="F283">
-        <v>200</v>
+        <v>66.12</v>
       </c>
       <c r="G283" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H283" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Seguro celular</v>
       </c>
     </row>
     <row r="284">
@@ -12557,22 +12557,22 @@
         <v>Setembro</v>
       </c>
       <c r="B284">
-        <v>46275</v>
+        <v>46280</v>
       </c>
       <c r="D284" t="str">
-        <v>Nu Seguro Celular</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E284" t="str">
-        <v>Serviços</v>
+        <v>Família</v>
       </c>
       <c r="F284">
-        <v>66.12</v>
+        <v>150</v>
       </c>
       <c r="G284" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H284" t="str">
-        <v>Seguro celular</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="285">
@@ -12580,22 +12580,22 @@
         <v>Setembro</v>
       </c>
       <c r="B285">
-        <v>46289</v>
+        <v>46285</v>
       </c>
       <c r="D285" t="str">
-        <v>Sócio Torcedor Flamengo</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E285" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Família</v>
       </c>
       <c r="F285">
-        <v>312</v>
+        <v>200</v>
       </c>
       <c r="G285" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H285" t="str">
-        <v>Sócio torcedor CRF</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="286">
@@ -12603,22 +12603,22 @@
         <v>Setembro</v>
       </c>
       <c r="B286">
-        <v>46289</v>
+        <v>46285</v>
       </c>
       <c r="D286" t="str">
-        <v>Netflix</v>
+        <v>YouTube Premium</v>
       </c>
       <c r="E286" t="str">
         <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F286">
-        <v>20.9</v>
+        <v>25.92</v>
       </c>
       <c r="G286" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H286" t="str">
-        <v>Assinatura Netflix</v>
+        <v>Assinatura YouTube</v>
       </c>
     </row>
     <row r="287">
@@ -12626,22 +12626,22 @@
         <v>Setembro</v>
       </c>
       <c r="B287">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="D287" t="str">
-        <v>YouTube Premium</v>
+        <v>Netflix</v>
       </c>
       <c r="E287" t="str">
         <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F287">
-        <v>25.92</v>
+        <v>20.9</v>
       </c>
       <c r="G287" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H287" t="str">
-        <v>Assinatura YouTube</v>
+        <v>Assinatura Netflix</v>
       </c>
     </row>
     <row r="288">
@@ -12669,25 +12669,25 @@
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>Setembro</v>
+        <v>Outubro</v>
       </c>
       <c r="B289">
-        <v>46275</v>
+        <v>46305</v>
       </c>
       <c r="D289" t="str">
-        <v>Condomínio Citta America</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
       </c>
       <c r="E289" t="str">
         <v>Moradia</v>
       </c>
       <c r="F289">
-        <v>51.6</v>
+        <v>1300</v>
       </c>
       <c r="G289" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H289" t="str">
-        <v>Taxa condomínio / garagem</v>
+        <v>Aluguel residencial parcela 1</v>
       </c>
     </row>
     <row r="290">
@@ -12695,22 +12695,22 @@
         <v>Outubro</v>
       </c>
       <c r="B290">
-        <v>46305</v>
+        <v>46320</v>
       </c>
       <c r="D290" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
       </c>
       <c r="E290" t="str">
         <v>Moradia</v>
       </c>
       <c r="F290">
-        <v>1300</v>
+        <v>700</v>
       </c>
       <c r="G290" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H290" t="str">
-        <v>Aluguel residencial parcela 1</v>
+        <v>Aluguel residencial parcela 2</v>
       </c>
     </row>
     <row r="291">
@@ -12718,22 +12718,22 @@
         <v>Outubro</v>
       </c>
       <c r="B291">
-        <v>46320</v>
+        <v>46305</v>
       </c>
       <c r="D291" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+        <v>IPTU (parcela mensal) Lusitania</v>
       </c>
       <c r="E291" t="str">
         <v>Moradia</v>
       </c>
       <c r="F291">
-        <v>700</v>
+        <v>290</v>
       </c>
       <c r="G291" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H291" t="str">
-        <v>Aluguel residencial parcela 2</v>
+        <v>Parcela IPTU residencial</v>
       </c>
     </row>
     <row r="292">
@@ -12741,22 +12741,22 @@
         <v>Outubro</v>
       </c>
       <c r="B292">
-        <v>46305</v>
+        <v>46300</v>
       </c>
       <c r="D292" t="str">
-        <v>IPTU (parcela mensal) Lusitania</v>
+        <v>Diarista / Limpeza - Semana 1 (2 diárias)</v>
       </c>
       <c r="E292" t="str">
         <v>Moradia</v>
       </c>
       <c r="F292">
-        <v>290</v>
+        <v>440</v>
       </c>
       <c r="G292" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H292" t="str">
-        <v>Parcela IPTU residencial</v>
+        <v>2 diárias de R$ 220 (Semana 1)</v>
       </c>
     </row>
     <row r="293">
@@ -12767,7 +12767,7 @@
         <v>46307</v>
       </c>
       <c r="D293" t="str">
-        <v>Diarista / Limpeza - Maria Auxiliadora (1/2)</v>
+        <v>Diarista / Limpeza - Semana 2 (2 diárias)</v>
       </c>
       <c r="E293" t="str">
         <v>Moradia</v>
@@ -12779,7 +12779,7 @@
         <v>⏳ Pendente</v>
       </c>
       <c r="H293" t="str">
-        <v>Diárias limpeza quinzena 1</v>
+        <v>2 diárias de R$ 220 (Semana 2)</v>
       </c>
     </row>
     <row r="294">
@@ -12787,22 +12787,22 @@
         <v>Outubro</v>
       </c>
       <c r="B294">
-        <v>46321</v>
+        <v>46314</v>
       </c>
       <c r="D294" t="str">
-        <v>Diarista / Limpeza - Maria Auxiliadora (2/2)</v>
+        <v>Diarista / Limpeza - Semana 3 (2 diárias)</v>
       </c>
       <c r="E294" t="str">
         <v>Moradia</v>
       </c>
       <c r="F294">
-        <v>220</v>
+        <v>440</v>
       </c>
       <c r="G294" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H294" t="str">
-        <v>Diária limpeza quinzena 2</v>
+        <v>2 diárias de R$ 220 (Semana 3)</v>
       </c>
     </row>
     <row r="295">
@@ -12813,19 +12813,19 @@
         <v>46321</v>
       </c>
       <c r="D295" t="str">
-        <v>Diarista / Limpeza - Rosana Francelino</v>
+        <v>Diarista / Limpeza - Semana 4 (2 diárias)</v>
       </c>
       <c r="E295" t="str">
         <v>Moradia</v>
       </c>
       <c r="F295">
-        <v>220</v>
+        <v>440</v>
       </c>
       <c r="G295" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H295" t="str">
-        <v>Diária limpeza quinzena 2</v>
+        <v>2 diárias de R$ 220 (Semana 4)</v>
       </c>
     </row>
     <row r="296">
@@ -12856,22 +12856,22 @@
         <v>Outubro</v>
       </c>
       <c r="B297">
-        <v>46310</v>
+        <v>46305</v>
       </c>
       <c r="D297" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>Nu Seguro Celular</v>
       </c>
       <c r="E297" t="str">
-        <v>Família</v>
+        <v>Serviços</v>
       </c>
       <c r="F297">
-        <v>150</v>
+        <v>66.12</v>
       </c>
       <c r="G297" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H297" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Seguro celular</v>
       </c>
     </row>
     <row r="298">
@@ -12879,7 +12879,7 @@
         <v>Outubro</v>
       </c>
       <c r="B298">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="D298" t="str">
         <v>Ajuda Familiar (Tia via Douglas)</v>
@@ -12888,7 +12888,7 @@
         <v>Família</v>
       </c>
       <c r="F298">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G298" t="str">
         <v>⏳ Pendente</v>
@@ -12902,22 +12902,22 @@
         <v>Outubro</v>
       </c>
       <c r="B299">
-        <v>46305</v>
+        <v>46315</v>
       </c>
       <c r="D299" t="str">
-        <v>Nu Seguro Celular</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E299" t="str">
-        <v>Serviços</v>
+        <v>Família</v>
       </c>
       <c r="F299">
-        <v>66.12</v>
+        <v>200</v>
       </c>
       <c r="G299" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H299" t="str">
-        <v>Seguro celular</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="300">
@@ -12925,22 +12925,22 @@
         <v>Outubro</v>
       </c>
       <c r="B300">
-        <v>46319</v>
+        <v>46315</v>
       </c>
       <c r="D300" t="str">
-        <v>Sócio Torcedor Flamengo</v>
+        <v>YouTube Premium</v>
       </c>
       <c r="E300" t="str">
         <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F300">
-        <v>312</v>
+        <v>25.92</v>
       </c>
       <c r="G300" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H300" t="str">
-        <v>Sócio torcedor CRF</v>
+        <v>Assinatura YouTube</v>
       </c>
     </row>
     <row r="301">
@@ -12971,68 +12971,68 @@
         <v>Outubro</v>
       </c>
       <c r="B302">
-        <v>46315</v>
+        <v>46297</v>
       </c>
       <c r="D302" t="str">
-        <v>YouTube Premium</v>
+        <v>Clube iFood</v>
       </c>
       <c r="E302" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Alimentação</v>
       </c>
       <c r="F302">
-        <v>25.92</v>
+        <v>5.95</v>
       </c>
       <c r="G302" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H302" t="str">
-        <v>Assinatura YouTube</v>
+        <v>Assinatura Clube iFood</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>Outubro</v>
+        <v>Novembro</v>
       </c>
       <c r="B303">
-        <v>46297</v>
+        <v>46336</v>
       </c>
       <c r="D303" t="str">
-        <v>Clube iFood</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
       </c>
       <c r="E303" t="str">
-        <v>Alimentação</v>
+        <v>Moradia</v>
       </c>
       <c r="F303">
-        <v>5.95</v>
+        <v>1300</v>
       </c>
       <c r="G303" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H303" t="str">
-        <v>Assinatura Clube iFood</v>
+        <v>Aluguel residencial parcela 1</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="str">
-        <v>Outubro</v>
+        <v>Novembro</v>
       </c>
       <c r="B304">
-        <v>46305</v>
+        <v>46351</v>
       </c>
       <c r="D304" t="str">
-        <v>Condomínio Citta America</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
       </c>
       <c r="E304" t="str">
         <v>Moradia</v>
       </c>
       <c r="F304">
-        <v>51.6</v>
+        <v>700</v>
       </c>
       <c r="G304" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H304" t="str">
-        <v>Taxa condomínio / garagem</v>
+        <v>Aluguel residencial parcela 2</v>
       </c>
     </row>
     <row r="305">
@@ -13043,19 +13043,19 @@
         <v>46336</v>
       </c>
       <c r="D305" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+        <v>IPTU (parcela mensal) Lusitania</v>
       </c>
       <c r="E305" t="str">
         <v>Moradia</v>
       </c>
       <c r="F305">
-        <v>1300</v>
+        <v>290</v>
       </c>
       <c r="G305" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H305" t="str">
-        <v>Aluguel residencial parcela 1</v>
+        <v>Parcela IPTU residencial</v>
       </c>
     </row>
     <row r="306">
@@ -13063,22 +13063,22 @@
         <v>Novembro</v>
       </c>
       <c r="B306">
-        <v>46351</v>
+        <v>46331</v>
       </c>
       <c r="D306" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+        <v>Diarista / Limpeza - Semana 1 (2 diárias)</v>
       </c>
       <c r="E306" t="str">
         <v>Moradia</v>
       </c>
       <c r="F306">
-        <v>700</v>
+        <v>440</v>
       </c>
       <c r="G306" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H306" t="str">
-        <v>Aluguel residencial parcela 2</v>
+        <v>2 diárias de R$ 220 (Semana 1)</v>
       </c>
     </row>
     <row r="307">
@@ -13086,22 +13086,22 @@
         <v>Novembro</v>
       </c>
       <c r="B307">
-        <v>46336</v>
+        <v>46338</v>
       </c>
       <c r="D307" t="str">
-        <v>IPTU (parcela mensal) Lusitania</v>
+        <v>Diarista / Limpeza - Semana 2 (2 diárias)</v>
       </c>
       <c r="E307" t="str">
         <v>Moradia</v>
       </c>
       <c r="F307">
-        <v>290</v>
+        <v>440</v>
       </c>
       <c r="G307" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H307" t="str">
-        <v>Parcela IPTU residencial</v>
+        <v>2 diárias de R$ 220 (Semana 2)</v>
       </c>
     </row>
     <row r="308">
@@ -13109,10 +13109,10 @@
         <v>Novembro</v>
       </c>
       <c r="B308">
-        <v>46338</v>
+        <v>46345</v>
       </c>
       <c r="D308" t="str">
-        <v>Diarista / Limpeza - Maria Auxiliadora (1/2)</v>
+        <v>Diarista / Limpeza - Semana 3 (2 diárias)</v>
       </c>
       <c r="E308" t="str">
         <v>Moradia</v>
@@ -13124,7 +13124,7 @@
         <v>⏳ Pendente</v>
       </c>
       <c r="H308" t="str">
-        <v>Diárias limpeza quinzena 1</v>
+        <v>2 diárias de R$ 220 (Semana 3)</v>
       </c>
     </row>
     <row r="309">
@@ -13135,19 +13135,19 @@
         <v>46352</v>
       </c>
       <c r="D309" t="str">
-        <v>Diarista / Limpeza - Maria Auxiliadora (2/2)</v>
+        <v>Diarista / Limpeza - Semana 4 (2 diárias)</v>
       </c>
       <c r="E309" t="str">
         <v>Moradia</v>
       </c>
       <c r="F309">
-        <v>220</v>
+        <v>440</v>
       </c>
       <c r="G309" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H309" t="str">
-        <v>Diária limpeza quinzena 2</v>
+        <v>2 diárias de R$ 220 (Semana 4)</v>
       </c>
     </row>
     <row r="310">
@@ -13155,22 +13155,22 @@
         <v>Novembro</v>
       </c>
       <c r="B310">
-        <v>46352</v>
+        <v>46331</v>
       </c>
       <c r="D310" t="str">
-        <v>Diarista / Limpeza - Rosana Francelino</v>
+        <v>Vivo Telefonia &amp; Internet</v>
       </c>
       <c r="E310" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F310">
-        <v>220</v>
+        <v>481.63</v>
       </c>
       <c r="G310" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H310" t="str">
-        <v>Diária limpeza quinzena 2</v>
+        <v>Linha celular e internet residencial</v>
       </c>
     </row>
     <row r="311">
@@ -13178,22 +13178,22 @@
         <v>Novembro</v>
       </c>
       <c r="B311">
-        <v>46331</v>
+        <v>46336</v>
       </c>
       <c r="D311" t="str">
-        <v>Vivo Telefonia &amp; Internet</v>
+        <v>Nu Seguro Celular</v>
       </c>
       <c r="E311" t="str">
         <v>Serviços</v>
       </c>
       <c r="F311">
-        <v>481.63</v>
+        <v>66.12</v>
       </c>
       <c r="G311" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H311" t="str">
-        <v>Linha celular e internet residencial</v>
+        <v>Seguro celular</v>
       </c>
     </row>
     <row r="312">
@@ -13247,22 +13247,22 @@
         <v>Novembro</v>
       </c>
       <c r="B314">
-        <v>46336</v>
+        <v>46346</v>
       </c>
       <c r="D314" t="str">
-        <v>Nu Seguro Celular</v>
+        <v>YouTube Premium</v>
       </c>
       <c r="E314" t="str">
-        <v>Serviços</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F314">
-        <v>66.12</v>
+        <v>25.92</v>
       </c>
       <c r="G314" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H314" t="str">
-        <v>Seguro celular</v>
+        <v>Assinatura YouTube</v>
       </c>
     </row>
     <row r="315">
@@ -13273,19 +13273,19 @@
         <v>46350</v>
       </c>
       <c r="D315" t="str">
-        <v>Sócio Torcedor Flamengo</v>
+        <v>Netflix</v>
       </c>
       <c r="E315" t="str">
         <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F315">
-        <v>312</v>
+        <v>20.9</v>
       </c>
       <c r="G315" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H315" t="str">
-        <v>Sócio torcedor CRF</v>
+        <v>Assinatura Netflix</v>
       </c>
     </row>
     <row r="316">
@@ -13293,91 +13293,91 @@
         <v>Novembro</v>
       </c>
       <c r="B316">
-        <v>46350</v>
+        <v>46328</v>
       </c>
       <c r="D316" t="str">
-        <v>Netflix</v>
+        <v>Clube iFood</v>
       </c>
       <c r="E316" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Alimentação</v>
       </c>
       <c r="F316">
-        <v>20.9</v>
+        <v>5.95</v>
       </c>
       <c r="G316" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H316" t="str">
-        <v>Assinatura Netflix</v>
+        <v>Assinatura Clube iFood</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B317">
-        <v>46346</v>
+        <v>46366</v>
       </c>
       <c r="D317" t="str">
-        <v>YouTube Premium</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
       </c>
       <c r="E317" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Moradia</v>
       </c>
       <c r="F317">
-        <v>25.92</v>
+        <v>1300</v>
       </c>
       <c r="G317" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H317" t="str">
-        <v>Assinatura YouTube</v>
+        <v>Aluguel residencial parcela 1</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B318">
-        <v>46328</v>
+        <v>46381</v>
       </c>
       <c r="D318" t="str">
-        <v>Clube iFood</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
       </c>
       <c r="E318" t="str">
-        <v>Alimentação</v>
+        <v>Moradia</v>
       </c>
       <c r="F318">
-        <v>5.95</v>
+        <v>700</v>
       </c>
       <c r="G318" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H318" t="str">
-        <v>Assinatura Clube iFood</v>
+        <v>Aluguel residencial parcela 2</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B319">
-        <v>46336</v>
+        <v>46366</v>
       </c>
       <c r="D319" t="str">
-        <v>Condomínio Citta America</v>
+        <v>IPTU (parcela mensal) Lusitania</v>
       </c>
       <c r="E319" t="str">
         <v>Moradia</v>
       </c>
       <c r="F319">
-        <v>51.6</v>
+        <v>290</v>
       </c>
       <c r="G319" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H319" t="str">
-        <v>Taxa condomínio / garagem</v>
+        <v>Parcela IPTU residencial</v>
       </c>
     </row>
     <row r="320">
@@ -13385,22 +13385,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B320">
-        <v>46366</v>
+        <v>46361</v>
       </c>
       <c r="D320" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+        <v>Diarista / Limpeza - Semana 1 (2 diárias)</v>
       </c>
       <c r="E320" t="str">
         <v>Moradia</v>
       </c>
       <c r="F320">
-        <v>1300</v>
+        <v>440</v>
       </c>
       <c r="G320" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H320" t="str">
-        <v>Aluguel residencial parcela 1</v>
+        <v>2 diárias de R$ 220 (Semana 1)</v>
       </c>
     </row>
     <row r="321">
@@ -13408,22 +13408,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B321">
-        <v>46381</v>
+        <v>46368</v>
       </c>
       <c r="D321" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+        <v>Diarista / Limpeza - Semana 2 (2 diárias)</v>
       </c>
       <c r="E321" t="str">
         <v>Moradia</v>
       </c>
       <c r="F321">
-        <v>700</v>
+        <v>440</v>
       </c>
       <c r="G321" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H321" t="str">
-        <v>Aluguel residencial parcela 2</v>
+        <v>2 diárias de R$ 220 (Semana 2)</v>
       </c>
     </row>
     <row r="322">
@@ -13431,22 +13431,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B322">
-        <v>46366</v>
+        <v>46375</v>
       </c>
       <c r="D322" t="str">
-        <v>IPTU (parcela mensal) Lusitania</v>
+        <v>Diarista / Limpeza - Semana 3 (2 diárias)</v>
       </c>
       <c r="E322" t="str">
         <v>Moradia</v>
       </c>
       <c r="F322">
-        <v>290</v>
+        <v>440</v>
       </c>
       <c r="G322" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H322" t="str">
-        <v>Parcela IPTU residencial</v>
+        <v>2 diárias de R$ 220 (Semana 3)</v>
       </c>
     </row>
     <row r="323">
@@ -13454,10 +13454,10 @@
         <v>Dezembro</v>
       </c>
       <c r="B323">
-        <v>46368</v>
+        <v>46382</v>
       </c>
       <c r="D323" t="str">
-        <v>Diarista / Limpeza - Maria Auxiliadora (1/2)</v>
+        <v>Diarista / Limpeza - Semana 4 (2 diárias)</v>
       </c>
       <c r="E323" t="str">
         <v>Moradia</v>
@@ -13469,7 +13469,7 @@
         <v>⏳ Pendente</v>
       </c>
       <c r="H323" t="str">
-        <v>Diárias limpeza quinzena 1</v>
+        <v>2 diárias de R$ 220 (Semana 4)</v>
       </c>
     </row>
     <row r="324">
@@ -13477,22 +13477,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B324">
-        <v>46382</v>
+        <v>46361</v>
       </c>
       <c r="D324" t="str">
-        <v>Diarista / Limpeza - Maria Auxiliadora (2/2)</v>
+        <v>Vivo Telefonia &amp; Internet</v>
       </c>
       <c r="E324" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F324">
-        <v>220</v>
+        <v>481.63</v>
       </c>
       <c r="G324" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H324" t="str">
-        <v>Diária limpeza quinzena 2</v>
+        <v>Linha celular e internet residencial</v>
       </c>
     </row>
     <row r="325">
@@ -13500,22 +13500,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B325">
-        <v>46382</v>
+        <v>46366</v>
       </c>
       <c r="D325" t="str">
-        <v>Diarista / Limpeza - Rosana Francelino</v>
+        <v>Nu Seguro Celular</v>
       </c>
       <c r="E325" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F325">
-        <v>220</v>
+        <v>66.12</v>
       </c>
       <c r="G325" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H325" t="str">
-        <v>Diária limpeza quinzena 2</v>
+        <v>Seguro celular</v>
       </c>
     </row>
     <row r="326">
@@ -13523,22 +13523,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B326">
-        <v>46361</v>
+        <v>46371</v>
       </c>
       <c r="D326" t="str">
-        <v>Vivo Telefonia &amp; Internet</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E326" t="str">
-        <v>Serviços</v>
+        <v>Família</v>
       </c>
       <c r="F326">
-        <v>481.63</v>
+        <v>150</v>
       </c>
       <c r="G326" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H326" t="str">
-        <v>Linha celular e internet residencial</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="327">
@@ -13546,7 +13546,7 @@
         <v>Dezembro</v>
       </c>
       <c r="B327">
-        <v>46371</v>
+        <v>46376</v>
       </c>
       <c r="D327" t="str">
         <v>Ajuda Familiar (Tia via Douglas)</v>
@@ -13555,7 +13555,7 @@
         <v>Família</v>
       </c>
       <c r="F327">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="G327" t="str">
         <v>⏳ Pendente</v>
@@ -13572,19 +13572,19 @@
         <v>46376</v>
       </c>
       <c r="D328" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>YouTube Premium</v>
       </c>
       <c r="E328" t="str">
-        <v>Família</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F328">
-        <v>200</v>
+        <v>25.92</v>
       </c>
       <c r="G328" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H328" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Assinatura YouTube</v>
       </c>
     </row>
     <row r="329">
@@ -13592,22 +13592,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B329">
-        <v>46366</v>
+        <v>46380</v>
       </c>
       <c r="D329" t="str">
-        <v>Nu Seguro Celular</v>
+        <v>Netflix</v>
       </c>
       <c r="E329" t="str">
-        <v>Serviços</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F329">
-        <v>66.12</v>
+        <v>20.9</v>
       </c>
       <c r="G329" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H329" t="str">
-        <v>Seguro celular</v>
+        <v>Assinatura Netflix</v>
       </c>
     </row>
     <row r="330">
@@ -13615,143 +13615,51 @@
         <v>Dezembro</v>
       </c>
       <c r="B330">
-        <v>46380</v>
+        <v>46358</v>
       </c>
       <c r="D330" t="str">
-        <v>Sócio Torcedor Flamengo</v>
+        <v>Clube iFood</v>
       </c>
       <c r="E330" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Alimentação</v>
       </c>
       <c r="F330">
-        <v>312</v>
+        <v>5.95</v>
       </c>
       <c r="G330" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H330" t="str">
-        <v>Sócio torcedor CRF</v>
+        <v>Assinatura Clube iFood</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B331">
-        <v>46380</v>
-      </c>
-      <c r="D331" t="str">
-        <v>Netflix</v>
-      </c>
-      <c r="E331" t="str">
-        <v>Lazer &amp; Assinaturas</v>
-      </c>
-      <c r="F331">
-        <v>20.9</v>
-      </c>
-      <c r="G331" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H331" t="str">
-        <v>Assinatura Netflix</v>
+        <v>Total</v>
+      </c>
+      <c r="D331">
+        <v>0</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B332">
-        <v>46376</v>
-      </c>
-      <c r="D332" t="str">
-        <v>YouTube Premium</v>
-      </c>
-      <c r="E332" t="str">
-        <v>Lazer &amp; Assinaturas</v>
-      </c>
-      <c r="F332">
-        <v>25.92</v>
-      </c>
-      <c r="G332" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H332" t="str">
-        <v>Assinatura YouTube</v>
+        <v>Total</v>
+      </c>
+      <c r="D332">
+        <v>415.18</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B333">
-        <v>46358</v>
-      </c>
-      <c r="D333" t="str">
-        <v>Clube iFood</v>
-      </c>
-      <c r="E333" t="str">
-        <v>Alimentação</v>
+        <v>💰 TOTAL GERAL PESSOAL</v>
       </c>
       <c r="F333">
-        <v>5.95</v>
-      </c>
-      <c r="G333" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H333" t="str">
-        <v>Assinatura Clube iFood</v>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B334">
-        <v>46366</v>
-      </c>
-      <c r="D334" t="str">
-        <v>Condomínio Citta America</v>
-      </c>
-      <c r="E334" t="str">
-        <v>Moradia</v>
-      </c>
-      <c r="F334">
-        <v>51.6</v>
-      </c>
-      <c r="G334" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H334" t="str">
-        <v>Taxa condomínio / garagem</v>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D335">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D336">
-        <v>415.18</v>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="str">
-        <v>💰 TOTAL GERAL PESSOAL</v>
-      </c>
-      <c r="F337">
         <v>2622.22</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H337"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H333"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ajuste diaristas quinzenais (2 diarias de R$ 220 por mes = R$ 440/mes)
</commit_message>
<xml_diff>
--- a/Controle_Financeiro_2026.xlsx
+++ b/Controle_Financeiro_2026.xlsx
@@ -786,16 +786,16 @@
         <v>0</v>
       </c>
       <c r="J14">
-        <v>4050</v>
+        <v>2730</v>
       </c>
       <c r="K14">
-        <v>4050</v>
+        <v>2730</v>
       </c>
       <c r="L14">
-        <v>4050</v>
+        <v>2730</v>
       </c>
       <c r="M14">
-        <v>4050</v>
+        <v>2730</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -1182,16 +1182,16 @@
         <v>7613.08</v>
       </c>
       <c r="J23">
-        <v>4997.52</v>
+        <v>3677.52</v>
       </c>
       <c r="K23">
-        <v>4997.52</v>
+        <v>3677.52</v>
       </c>
       <c r="L23">
-        <v>4997.52</v>
+        <v>3677.52</v>
       </c>
       <c r="M23">
-        <v>4997.52</v>
+        <v>3677.52</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -1231,16 +1231,16 @@
         <v>11867.75</v>
       </c>
       <c r="J26">
-        <v>6725.31</v>
+        <v>5405.31</v>
       </c>
       <c r="K26">
-        <v>6725.31</v>
+        <v>5405.31</v>
       </c>
       <c r="L26">
-        <v>6725.31</v>
+        <v>5405.31</v>
       </c>
       <c r="M26">
-        <v>6725.31</v>
+        <v>5405.31</v>
       </c>
       <c r="N26">
         <v>4220.7</v>
@@ -6394,7 +6394,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H333"/>
+  <dimension ref="A1:H325"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12419,22 +12419,22 @@
         <v>Setembro</v>
       </c>
       <c r="B278">
-        <v>46270</v>
+        <v>46277</v>
       </c>
       <c r="D278" t="str">
-        <v>Diarista / Limpeza - Semana 1 (2 diárias)</v>
+        <v>Diarista / Limpeza - Quinzena 1</v>
       </c>
       <c r="E278" t="str">
         <v>Moradia</v>
       </c>
       <c r="F278">
-        <v>440</v>
+        <v>220</v>
       </c>
       <c r="G278" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H278" t="str">
-        <v>2 diárias de R$ 220 (Semana 1)</v>
+        <v>1 diária (Quinzena 1)</v>
       </c>
     </row>
     <row r="279">
@@ -12442,22 +12442,22 @@
         <v>Setembro</v>
       </c>
       <c r="B279">
-        <v>46277</v>
+        <v>46291</v>
       </c>
       <c r="D279" t="str">
-        <v>Diarista / Limpeza - Semana 2 (2 diárias)</v>
+        <v>Diarista / Limpeza - Quinzena 2</v>
       </c>
       <c r="E279" t="str">
         <v>Moradia</v>
       </c>
       <c r="F279">
-        <v>440</v>
+        <v>220</v>
       </c>
       <c r="G279" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H279" t="str">
-        <v>2 diárias de R$ 220 (Semana 2)</v>
+        <v>1 diária (Quinzena 2)</v>
       </c>
     </row>
     <row r="280">
@@ -12465,22 +12465,22 @@
         <v>Setembro</v>
       </c>
       <c r="B280">
-        <v>46284</v>
+        <v>46270</v>
       </c>
       <c r="D280" t="str">
-        <v>Diarista / Limpeza - Semana 3 (2 diárias)</v>
+        <v>Vivo Telefonia &amp; Internet</v>
       </c>
       <c r="E280" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F280">
-        <v>440</v>
+        <v>481.63</v>
       </c>
       <c r="G280" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H280" t="str">
-        <v>2 diárias de R$ 220 (Semana 3)</v>
+        <v>Linha celular e internet residencial</v>
       </c>
     </row>
     <row r="281">
@@ -12488,22 +12488,22 @@
         <v>Setembro</v>
       </c>
       <c r="B281">
-        <v>46291</v>
+        <v>46275</v>
       </c>
       <c r="D281" t="str">
-        <v>Diarista / Limpeza - Semana 4 (2 diárias)</v>
+        <v>Nu Seguro Celular</v>
       </c>
       <c r="E281" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F281">
-        <v>440</v>
+        <v>66.12</v>
       </c>
       <c r="G281" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H281" t="str">
-        <v>2 diárias de R$ 220 (Semana 4)</v>
+        <v>Seguro celular</v>
       </c>
     </row>
     <row r="282">
@@ -12511,22 +12511,22 @@
         <v>Setembro</v>
       </c>
       <c r="B282">
-        <v>46270</v>
+        <v>46280</v>
       </c>
       <c r="D282" t="str">
-        <v>Vivo Telefonia &amp; Internet</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E282" t="str">
-        <v>Serviços</v>
+        <v>Família</v>
       </c>
       <c r="F282">
-        <v>481.63</v>
+        <v>150</v>
       </c>
       <c r="G282" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H282" t="str">
-        <v>Linha celular e internet residencial</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="283">
@@ -12534,22 +12534,22 @@
         <v>Setembro</v>
       </c>
       <c r="B283">
-        <v>46275</v>
+        <v>46285</v>
       </c>
       <c r="D283" t="str">
-        <v>Nu Seguro Celular</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E283" t="str">
-        <v>Serviços</v>
+        <v>Família</v>
       </c>
       <c r="F283">
-        <v>66.12</v>
+        <v>200</v>
       </c>
       <c r="G283" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H283" t="str">
-        <v>Seguro celular</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="284">
@@ -12557,22 +12557,22 @@
         <v>Setembro</v>
       </c>
       <c r="B284">
-        <v>46280</v>
+        <v>46285</v>
       </c>
       <c r="D284" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>YouTube Premium</v>
       </c>
       <c r="E284" t="str">
-        <v>Família</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F284">
-        <v>150</v>
+        <v>25.92</v>
       </c>
       <c r="G284" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H284" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Assinatura YouTube</v>
       </c>
     </row>
     <row r="285">
@@ -12580,22 +12580,22 @@
         <v>Setembro</v>
       </c>
       <c r="B285">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="D285" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>Netflix</v>
       </c>
       <c r="E285" t="str">
-        <v>Família</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F285">
-        <v>200</v>
+        <v>20.9</v>
       </c>
       <c r="G285" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H285" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Assinatura Netflix</v>
       </c>
     </row>
     <row r="286">
@@ -12603,68 +12603,68 @@
         <v>Setembro</v>
       </c>
       <c r="B286">
-        <v>46285</v>
+        <v>46267</v>
       </c>
       <c r="D286" t="str">
-        <v>YouTube Premium</v>
+        <v>Clube iFood</v>
       </c>
       <c r="E286" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Alimentação</v>
       </c>
       <c r="F286">
-        <v>25.92</v>
+        <v>5.95</v>
       </c>
       <c r="G286" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H286" t="str">
-        <v>Assinatura YouTube</v>
+        <v>Assinatura Clube iFood</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>Setembro</v>
+        <v>Outubro</v>
       </c>
       <c r="B287">
-        <v>46289</v>
+        <v>46305</v>
       </c>
       <c r="D287" t="str">
-        <v>Netflix</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
       </c>
       <c r="E287" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Moradia</v>
       </c>
       <c r="F287">
-        <v>20.9</v>
+        <v>1300</v>
       </c>
       <c r="G287" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H287" t="str">
-        <v>Assinatura Netflix</v>
+        <v>Aluguel residencial parcela 1</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>Setembro</v>
+        <v>Outubro</v>
       </c>
       <c r="B288">
-        <v>46267</v>
+        <v>46320</v>
       </c>
       <c r="D288" t="str">
-        <v>Clube iFood</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
       </c>
       <c r="E288" t="str">
-        <v>Alimentação</v>
+        <v>Moradia</v>
       </c>
       <c r="F288">
-        <v>5.95</v>
+        <v>700</v>
       </c>
       <c r="G288" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H288" t="str">
-        <v>Assinatura Clube iFood</v>
+        <v>Aluguel residencial parcela 2</v>
       </c>
     </row>
     <row r="289">
@@ -12675,19 +12675,19 @@
         <v>46305</v>
       </c>
       <c r="D289" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+        <v>IPTU (parcela mensal) Lusitania</v>
       </c>
       <c r="E289" t="str">
         <v>Moradia</v>
       </c>
       <c r="F289">
-        <v>1300</v>
+        <v>290</v>
       </c>
       <c r="G289" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H289" t="str">
-        <v>Aluguel residencial parcela 1</v>
+        <v>Parcela IPTU residencial</v>
       </c>
     </row>
     <row r="290">
@@ -12695,22 +12695,22 @@
         <v>Outubro</v>
       </c>
       <c r="B290">
-        <v>46320</v>
+        <v>46307</v>
       </c>
       <c r="D290" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+        <v>Diarista / Limpeza - Quinzena 1</v>
       </c>
       <c r="E290" t="str">
         <v>Moradia</v>
       </c>
       <c r="F290">
-        <v>700</v>
+        <v>220</v>
       </c>
       <c r="G290" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H290" t="str">
-        <v>Aluguel residencial parcela 2</v>
+        <v>1 diária (Quinzena 1)</v>
       </c>
     </row>
     <row r="291">
@@ -12718,22 +12718,22 @@
         <v>Outubro</v>
       </c>
       <c r="B291">
-        <v>46305</v>
+        <v>46321</v>
       </c>
       <c r="D291" t="str">
-        <v>IPTU (parcela mensal) Lusitania</v>
+        <v>Diarista / Limpeza - Quinzena 2</v>
       </c>
       <c r="E291" t="str">
         <v>Moradia</v>
       </c>
       <c r="F291">
-        <v>290</v>
+        <v>220</v>
       </c>
       <c r="G291" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H291" t="str">
-        <v>Parcela IPTU residencial</v>
+        <v>1 diária (Quinzena 2)</v>
       </c>
     </row>
     <row r="292">
@@ -12744,19 +12744,19 @@
         <v>46300</v>
       </c>
       <c r="D292" t="str">
-        <v>Diarista / Limpeza - Semana 1 (2 diárias)</v>
+        <v>Vivo Telefonia &amp; Internet</v>
       </c>
       <c r="E292" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F292">
-        <v>440</v>
+        <v>481.63</v>
       </c>
       <c r="G292" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H292" t="str">
-        <v>2 diárias de R$ 220 (Semana 1)</v>
+        <v>Linha celular e internet residencial</v>
       </c>
     </row>
     <row r="293">
@@ -12764,22 +12764,22 @@
         <v>Outubro</v>
       </c>
       <c r="B293">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="D293" t="str">
-        <v>Diarista / Limpeza - Semana 2 (2 diárias)</v>
+        <v>Nu Seguro Celular</v>
       </c>
       <c r="E293" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F293">
-        <v>440</v>
+        <v>66.12</v>
       </c>
       <c r="G293" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H293" t="str">
-        <v>2 diárias de R$ 220 (Semana 2)</v>
+        <v>Seguro celular</v>
       </c>
     </row>
     <row r="294">
@@ -12787,22 +12787,22 @@
         <v>Outubro</v>
       </c>
       <c r="B294">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="D294" t="str">
-        <v>Diarista / Limpeza - Semana 3 (2 diárias)</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E294" t="str">
-        <v>Moradia</v>
+        <v>Família</v>
       </c>
       <c r="F294">
-        <v>440</v>
+        <v>150</v>
       </c>
       <c r="G294" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H294" t="str">
-        <v>2 diárias de R$ 220 (Semana 3)</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="295">
@@ -12810,22 +12810,22 @@
         <v>Outubro</v>
       </c>
       <c r="B295">
-        <v>46321</v>
+        <v>46315</v>
       </c>
       <c r="D295" t="str">
-        <v>Diarista / Limpeza - Semana 4 (2 diárias)</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E295" t="str">
-        <v>Moradia</v>
+        <v>Família</v>
       </c>
       <c r="F295">
-        <v>440</v>
+        <v>200</v>
       </c>
       <c r="G295" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H295" t="str">
-        <v>2 diárias de R$ 220 (Semana 4)</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="296">
@@ -12833,22 +12833,22 @@
         <v>Outubro</v>
       </c>
       <c r="B296">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="D296" t="str">
-        <v>Vivo Telefonia &amp; Internet</v>
+        <v>YouTube Premium</v>
       </c>
       <c r="E296" t="str">
-        <v>Serviços</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F296">
-        <v>481.63</v>
+        <v>25.92</v>
       </c>
       <c r="G296" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H296" t="str">
-        <v>Linha celular e internet residencial</v>
+        <v>Assinatura YouTube</v>
       </c>
     </row>
     <row r="297">
@@ -12856,22 +12856,22 @@
         <v>Outubro</v>
       </c>
       <c r="B297">
-        <v>46305</v>
+        <v>46319</v>
       </c>
       <c r="D297" t="str">
-        <v>Nu Seguro Celular</v>
+        <v>Netflix</v>
       </c>
       <c r="E297" t="str">
-        <v>Serviços</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F297">
-        <v>66.12</v>
+        <v>20.9</v>
       </c>
       <c r="G297" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H297" t="str">
-        <v>Seguro celular</v>
+        <v>Assinatura Netflix</v>
       </c>
     </row>
     <row r="298">
@@ -12879,114 +12879,114 @@
         <v>Outubro</v>
       </c>
       <c r="B298">
-        <v>46310</v>
+        <v>46297</v>
       </c>
       <c r="D298" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>Clube iFood</v>
       </c>
       <c r="E298" t="str">
-        <v>Família</v>
+        <v>Alimentação</v>
       </c>
       <c r="F298">
-        <v>150</v>
+        <v>5.95</v>
       </c>
       <c r="G298" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H298" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Assinatura Clube iFood</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>Outubro</v>
+        <v>Novembro</v>
       </c>
       <c r="B299">
-        <v>46315</v>
+        <v>46336</v>
       </c>
       <c r="D299" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
       </c>
       <c r="E299" t="str">
-        <v>Família</v>
+        <v>Moradia</v>
       </c>
       <c r="F299">
-        <v>200</v>
+        <v>1300</v>
       </c>
       <c r="G299" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H299" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Aluguel residencial parcela 1</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="str">
-        <v>Outubro</v>
+        <v>Novembro</v>
       </c>
       <c r="B300">
-        <v>46315</v>
+        <v>46351</v>
       </c>
       <c r="D300" t="str">
-        <v>YouTube Premium</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
       </c>
       <c r="E300" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Moradia</v>
       </c>
       <c r="F300">
-        <v>25.92</v>
+        <v>700</v>
       </c>
       <c r="G300" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H300" t="str">
-        <v>Assinatura YouTube</v>
+        <v>Aluguel residencial parcela 2</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="str">
-        <v>Outubro</v>
+        <v>Novembro</v>
       </c>
       <c r="B301">
-        <v>46319</v>
+        <v>46336</v>
       </c>
       <c r="D301" t="str">
-        <v>Netflix</v>
+        <v>IPTU (parcela mensal) Lusitania</v>
       </c>
       <c r="E301" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Moradia</v>
       </c>
       <c r="F301">
-        <v>20.9</v>
+        <v>290</v>
       </c>
       <c r="G301" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H301" t="str">
-        <v>Assinatura Netflix</v>
+        <v>Parcela IPTU residencial</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="str">
-        <v>Outubro</v>
+        <v>Novembro</v>
       </c>
       <c r="B302">
-        <v>46297</v>
+        <v>46338</v>
       </c>
       <c r="D302" t="str">
-        <v>Clube iFood</v>
+        <v>Diarista / Limpeza - Quinzena 1</v>
       </c>
       <c r="E302" t="str">
-        <v>Alimentação</v>
+        <v>Moradia</v>
       </c>
       <c r="F302">
-        <v>5.95</v>
+        <v>220</v>
       </c>
       <c r="G302" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H302" t="str">
-        <v>Assinatura Clube iFood</v>
+        <v>1 diária (Quinzena 1)</v>
       </c>
     </row>
     <row r="303">
@@ -12994,22 +12994,22 @@
         <v>Novembro</v>
       </c>
       <c r="B303">
-        <v>46336</v>
+        <v>46352</v>
       </c>
       <c r="D303" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+        <v>Diarista / Limpeza - Quinzena 2</v>
       </c>
       <c r="E303" t="str">
         <v>Moradia</v>
       </c>
       <c r="F303">
-        <v>1300</v>
+        <v>220</v>
       </c>
       <c r="G303" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H303" t="str">
-        <v>Aluguel residencial parcela 1</v>
+        <v>1 diária (Quinzena 2)</v>
       </c>
     </row>
     <row r="304">
@@ -13017,22 +13017,22 @@
         <v>Novembro</v>
       </c>
       <c r="B304">
-        <v>46351</v>
+        <v>46331</v>
       </c>
       <c r="D304" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+        <v>Vivo Telefonia &amp; Internet</v>
       </c>
       <c r="E304" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F304">
-        <v>700</v>
+        <v>481.63</v>
       </c>
       <c r="G304" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H304" t="str">
-        <v>Aluguel residencial parcela 2</v>
+        <v>Linha celular e internet residencial</v>
       </c>
     </row>
     <row r="305">
@@ -13043,19 +13043,19 @@
         <v>46336</v>
       </c>
       <c r="D305" t="str">
-        <v>IPTU (parcela mensal) Lusitania</v>
+        <v>Nu Seguro Celular</v>
       </c>
       <c r="E305" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F305">
-        <v>290</v>
+        <v>66.12</v>
       </c>
       <c r="G305" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H305" t="str">
-        <v>Parcela IPTU residencial</v>
+        <v>Seguro celular</v>
       </c>
     </row>
     <row r="306">
@@ -13063,22 +13063,22 @@
         <v>Novembro</v>
       </c>
       <c r="B306">
-        <v>46331</v>
+        <v>46341</v>
       </c>
       <c r="D306" t="str">
-        <v>Diarista / Limpeza - Semana 1 (2 diárias)</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E306" t="str">
-        <v>Moradia</v>
+        <v>Família</v>
       </c>
       <c r="F306">
-        <v>440</v>
+        <v>150</v>
       </c>
       <c r="G306" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H306" t="str">
-        <v>2 diárias de R$ 220 (Semana 1)</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="307">
@@ -13086,22 +13086,22 @@
         <v>Novembro</v>
       </c>
       <c r="B307">
-        <v>46338</v>
+        <v>46346</v>
       </c>
       <c r="D307" t="str">
-        <v>Diarista / Limpeza - Semana 2 (2 diárias)</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E307" t="str">
-        <v>Moradia</v>
+        <v>Família</v>
       </c>
       <c r="F307">
-        <v>440</v>
+        <v>200</v>
       </c>
       <c r="G307" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H307" t="str">
-        <v>2 diárias de R$ 220 (Semana 2)</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="308">
@@ -13109,22 +13109,22 @@
         <v>Novembro</v>
       </c>
       <c r="B308">
-        <v>46345</v>
+        <v>46346</v>
       </c>
       <c r="D308" t="str">
-        <v>Diarista / Limpeza - Semana 3 (2 diárias)</v>
+        <v>YouTube Premium</v>
       </c>
       <c r="E308" t="str">
-        <v>Moradia</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F308">
-        <v>440</v>
+        <v>25.92</v>
       </c>
       <c r="G308" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H308" t="str">
-        <v>2 diárias de R$ 220 (Semana 3)</v>
+        <v>Assinatura YouTube</v>
       </c>
     </row>
     <row r="309">
@@ -13132,22 +13132,22 @@
         <v>Novembro</v>
       </c>
       <c r="B309">
-        <v>46352</v>
+        <v>46350</v>
       </c>
       <c r="D309" t="str">
-        <v>Diarista / Limpeza - Semana 4 (2 diárias)</v>
+        <v>Netflix</v>
       </c>
       <c r="E309" t="str">
-        <v>Moradia</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F309">
-        <v>440</v>
+        <v>20.9</v>
       </c>
       <c r="G309" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H309" t="str">
-        <v>2 diárias de R$ 220 (Semana 4)</v>
+        <v>Assinatura Netflix</v>
       </c>
     </row>
     <row r="310">
@@ -13155,160 +13155,160 @@
         <v>Novembro</v>
       </c>
       <c r="B310">
-        <v>46331</v>
+        <v>46328</v>
       </c>
       <c r="D310" t="str">
-        <v>Vivo Telefonia &amp; Internet</v>
+        <v>Clube iFood</v>
       </c>
       <c r="E310" t="str">
-        <v>Serviços</v>
+        <v>Alimentação</v>
       </c>
       <c r="F310">
-        <v>481.63</v>
+        <v>5.95</v>
       </c>
       <c r="G310" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H310" t="str">
-        <v>Linha celular e internet residencial</v>
+        <v>Assinatura Clube iFood</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B311">
-        <v>46336</v>
+        <v>46366</v>
       </c>
       <c r="D311" t="str">
-        <v>Nu Seguro Celular</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
       </c>
       <c r="E311" t="str">
-        <v>Serviços</v>
+        <v>Moradia</v>
       </c>
       <c r="F311">
-        <v>66.12</v>
+        <v>1300</v>
       </c>
       <c r="G311" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H311" t="str">
-        <v>Seguro celular</v>
+        <v>Aluguel residencial parcela 1</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B312">
-        <v>46341</v>
+        <v>46381</v>
       </c>
       <c r="D312" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
       </c>
       <c r="E312" t="str">
-        <v>Família</v>
+        <v>Moradia</v>
       </c>
       <c r="F312">
-        <v>150</v>
+        <v>700</v>
       </c>
       <c r="G312" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H312" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Aluguel residencial parcela 2</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B313">
-        <v>46346</v>
+        <v>46366</v>
       </c>
       <c r="D313" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
+        <v>IPTU (parcela mensal) Lusitania</v>
       </c>
       <c r="E313" t="str">
-        <v>Família</v>
+        <v>Moradia</v>
       </c>
       <c r="F313">
-        <v>200</v>
+        <v>290</v>
       </c>
       <c r="G313" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H313" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
+        <v>Parcela IPTU residencial</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B314">
-        <v>46346</v>
+        <v>46368</v>
       </c>
       <c r="D314" t="str">
-        <v>YouTube Premium</v>
+        <v>Diarista / Limpeza - Quinzena 1</v>
       </c>
       <c r="E314" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Moradia</v>
       </c>
       <c r="F314">
-        <v>25.92</v>
+        <v>220</v>
       </c>
       <c r="G314" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H314" t="str">
-        <v>Assinatura YouTube</v>
+        <v>1 diária (Quinzena 1)</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B315">
-        <v>46350</v>
+        <v>46382</v>
       </c>
       <c r="D315" t="str">
-        <v>Netflix</v>
+        <v>Diarista / Limpeza - Quinzena 2</v>
       </c>
       <c r="E315" t="str">
-        <v>Lazer &amp; Assinaturas</v>
+        <v>Moradia</v>
       </c>
       <c r="F315">
-        <v>20.9</v>
+        <v>220</v>
       </c>
       <c r="G315" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H315" t="str">
-        <v>Assinatura Netflix</v>
+        <v>1 diária (Quinzena 2)</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>Novembro</v>
+        <v>Dezembro</v>
       </c>
       <c r="B316">
-        <v>46328</v>
+        <v>46361</v>
       </c>
       <c r="D316" t="str">
-        <v>Clube iFood</v>
+        <v>Vivo Telefonia &amp; Internet</v>
       </c>
       <c r="E316" t="str">
-        <v>Alimentação</v>
+        <v>Serviços</v>
       </c>
       <c r="F316">
-        <v>5.95</v>
+        <v>481.63</v>
       </c>
       <c r="G316" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H316" t="str">
-        <v>Assinatura Clube iFood</v>
+        <v>Linha celular e internet residencial</v>
       </c>
     </row>
     <row r="317">
@@ -13319,19 +13319,19 @@
         <v>46366</v>
       </c>
       <c r="D317" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (1/2)</v>
+        <v>Nu Seguro Celular</v>
       </c>
       <c r="E317" t="str">
-        <v>Moradia</v>
+        <v>Serviços</v>
       </c>
       <c r="F317">
-        <v>1300</v>
+        <v>66.12</v>
       </c>
       <c r="G317" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H317" t="str">
-        <v>Aluguel residencial parcela 1</v>
+        <v>Seguro celular</v>
       </c>
     </row>
     <row r="318">
@@ -13339,22 +13339,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B318">
-        <v>46381</v>
+        <v>46371</v>
       </c>
       <c r="D318" t="str">
-        <v>Aluguel Moradia e afins - Lucian Balin (2/2)</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E318" t="str">
-        <v>Moradia</v>
+        <v>Família</v>
       </c>
       <c r="F318">
-        <v>700</v>
+        <v>150</v>
       </c>
       <c r="G318" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H318" t="str">
-        <v>Aluguel residencial parcela 2</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="319">
@@ -13362,22 +13362,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B319">
-        <v>46366</v>
+        <v>46376</v>
       </c>
       <c r="D319" t="str">
-        <v>IPTU (parcela mensal) Lusitania</v>
+        <v>Ajuda Familiar (Tia via Douglas)</v>
       </c>
       <c r="E319" t="str">
-        <v>Moradia</v>
+        <v>Família</v>
       </c>
       <c r="F319">
-        <v>290</v>
+        <v>200</v>
       </c>
       <c r="G319" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H319" t="str">
-        <v>Parcela IPTU residencial</v>
+        <v>Dinheiro enviado para a Tia via Douglas</v>
       </c>
     </row>
     <row r="320">
@@ -13385,22 +13385,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B320">
-        <v>46361</v>
+        <v>46376</v>
       </c>
       <c r="D320" t="str">
-        <v>Diarista / Limpeza - Semana 1 (2 diárias)</v>
+        <v>YouTube Premium</v>
       </c>
       <c r="E320" t="str">
-        <v>Moradia</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F320">
-        <v>440</v>
+        <v>25.92</v>
       </c>
       <c r="G320" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H320" t="str">
-        <v>2 diárias de R$ 220 (Semana 1)</v>
+        <v>Assinatura YouTube</v>
       </c>
     </row>
     <row r="321">
@@ -13408,22 +13408,22 @@
         <v>Dezembro</v>
       </c>
       <c r="B321">
-        <v>46368</v>
+        <v>46380</v>
       </c>
       <c r="D321" t="str">
-        <v>Diarista / Limpeza - Semana 2 (2 diárias)</v>
+        <v>Netflix</v>
       </c>
       <c r="E321" t="str">
-        <v>Moradia</v>
+        <v>Lazer &amp; Assinaturas</v>
       </c>
       <c r="F321">
-        <v>440</v>
+        <v>20.9</v>
       </c>
       <c r="G321" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H321" t="str">
-        <v>2 diárias de R$ 220 (Semana 2)</v>
+        <v>Assinatura Netflix</v>
       </c>
     </row>
     <row r="322">
@@ -13431,235 +13431,51 @@
         <v>Dezembro</v>
       </c>
       <c r="B322">
-        <v>46375</v>
+        <v>46358</v>
       </c>
       <c r="D322" t="str">
-        <v>Diarista / Limpeza - Semana 3 (2 diárias)</v>
+        <v>Clube iFood</v>
       </c>
       <c r="E322" t="str">
-        <v>Moradia</v>
+        <v>Alimentação</v>
       </c>
       <c r="F322">
-        <v>440</v>
+        <v>5.95</v>
       </c>
       <c r="G322" t="str">
         <v>⏳ Pendente</v>
       </c>
       <c r="H322" t="str">
-        <v>2 diárias de R$ 220 (Semana 3)</v>
+        <v>Assinatura Clube iFood</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B323">
-        <v>46382</v>
-      </c>
-      <c r="D323" t="str">
-        <v>Diarista / Limpeza - Semana 4 (2 diárias)</v>
-      </c>
-      <c r="E323" t="str">
-        <v>Moradia</v>
-      </c>
-      <c r="F323">
-        <v>440</v>
-      </c>
-      <c r="G323" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H323" t="str">
-        <v>2 diárias de R$ 220 (Semana 4)</v>
+        <v>Total</v>
+      </c>
+      <c r="D323">
+        <v>0</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B324">
-        <v>46361</v>
-      </c>
-      <c r="D324" t="str">
-        <v>Vivo Telefonia &amp; Internet</v>
-      </c>
-      <c r="E324" t="str">
-        <v>Serviços</v>
-      </c>
-      <c r="F324">
-        <v>481.63</v>
-      </c>
-      <c r="G324" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H324" t="str">
-        <v>Linha celular e internet residencial</v>
+        <v>Total</v>
+      </c>
+      <c r="D324">
+        <v>415.18</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B325">
-        <v>46366</v>
-      </c>
-      <c r="D325" t="str">
-        <v>Nu Seguro Celular</v>
-      </c>
-      <c r="E325" t="str">
-        <v>Serviços</v>
+        <v>💰 TOTAL GERAL PESSOAL</v>
       </c>
       <c r="F325">
-        <v>66.12</v>
-      </c>
-      <c r="G325" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H325" t="str">
-        <v>Seguro celular</v>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B326">
-        <v>46371</v>
-      </c>
-      <c r="D326" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
-      </c>
-      <c r="E326" t="str">
-        <v>Família</v>
-      </c>
-      <c r="F326">
-        <v>150</v>
-      </c>
-      <c r="G326" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H326" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B327">
-        <v>46376</v>
-      </c>
-      <c r="D327" t="str">
-        <v>Ajuda Familiar (Tia via Douglas)</v>
-      </c>
-      <c r="E327" t="str">
-        <v>Família</v>
-      </c>
-      <c r="F327">
-        <v>200</v>
-      </c>
-      <c r="G327" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H327" t="str">
-        <v>Dinheiro enviado para a Tia via Douglas</v>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B328">
-        <v>46376</v>
-      </c>
-      <c r="D328" t="str">
-        <v>YouTube Premium</v>
-      </c>
-      <c r="E328" t="str">
-        <v>Lazer &amp; Assinaturas</v>
-      </c>
-      <c r="F328">
-        <v>25.92</v>
-      </c>
-      <c r="G328" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H328" t="str">
-        <v>Assinatura YouTube</v>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B329">
-        <v>46380</v>
-      </c>
-      <c r="D329" t="str">
-        <v>Netflix</v>
-      </c>
-      <c r="E329" t="str">
-        <v>Lazer &amp; Assinaturas</v>
-      </c>
-      <c r="F329">
-        <v>20.9</v>
-      </c>
-      <c r="G329" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H329" t="str">
-        <v>Assinatura Netflix</v>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="str">
-        <v>Dezembro</v>
-      </c>
-      <c r="B330">
-        <v>46358</v>
-      </c>
-      <c r="D330" t="str">
-        <v>Clube iFood</v>
-      </c>
-      <c r="E330" t="str">
-        <v>Alimentação</v>
-      </c>
-      <c r="F330">
-        <v>5.95</v>
-      </c>
-      <c r="G330" t="str">
-        <v>⏳ Pendente</v>
-      </c>
-      <c r="H330" t="str">
-        <v>Assinatura Clube iFood</v>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D331">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="str">
-        <v>Total</v>
-      </c>
-      <c r="D332">
-        <v>415.18</v>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="str">
-        <v>💰 TOTAL GERAL PESSOAL</v>
-      </c>
-      <c r="F333">
         <v>2622.22</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H333"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H325"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>